<commit_message>
rebuild the pipeline on the blood-filtered 1902-protein matrix
</commit_message>
<xml_diff>
--- a/04_Figures/F05_prediction/WGCNA/continuous/c_data/cont_source_data.xlsx
+++ b/04_Figures/F05_prediction/WGCNA/continuous/c_data/cont_source_data.xlsx
@@ -531,28 +531,28 @@
         <v>15</v>
       </c>
       <c r="F2" t="n">
-        <v>-1.81251663533358</v>
+        <v>-0.283043144118497</v>
       </c>
       <c r="G2" t="n">
-        <v>14.4022727154361</v>
+        <v>9.72756430736979</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.528571428571428</v>
+        <v>-0.925</v>
       </c>
       <c r="I2" t="n">
-        <v>0.860696517412935</v>
+        <v>0.328358208955224</v>
       </c>
       <c r="J2" t="n">
-        <v>0.860696517412935</v>
+        <v>0.328358208955224</v>
       </c>
       <c r="K2" t="n">
-        <v>0.497512437810945</v>
+        <v>0.721393034825871</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.994880096982243</v>
+        <v>-0.821899082888611</v>
       </c>
       <c r="M2" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="3">
@@ -572,28 +572,28 @@
         <v>15</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.147959183673469</v>
+        <v>-0.280916645332961</v>
       </c>
       <c r="G3" t="n">
-        <v>1525.19203279155</v>
+        <v>1611.09718649317</v>
       </c>
       <c r="H3" t="n">
-        <v>-1</v>
+        <v>-0.978571428571428</v>
       </c>
       <c r="I3" t="n">
-        <v>0.154228855721393</v>
+        <v>0.343283582089552</v>
       </c>
       <c r="J3" t="n">
-        <v>0.159203980099502</v>
+        <v>0.343283582089552</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>0.810945273631841</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.998054416503016</v>
+        <v>-0.781938839178765</v>
       </c>
       <c r="M3" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="4">
@@ -613,28 +613,28 @@
         <v>15</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.855029298195405</v>
+        <v>-0.260891252068036</v>
       </c>
       <c r="G4" t="n">
-        <v>1811.95414955146</v>
+        <v>1493.86252645555</v>
       </c>
       <c r="H4" t="n">
-        <v>-1</v>
+        <v>-0.857142857142857</v>
       </c>
       <c r="I4" t="n">
-        <v>0.522388059701492</v>
+        <v>0.308457711442786</v>
       </c>
       <c r="J4" t="n">
-        <v>0.522388059701492</v>
+        <v>0.308457711442786</v>
       </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>0.63681592039801</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.931876560276423</v>
+        <v>-0.764766232416347</v>
       </c>
       <c r="M4" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="5">
@@ -654,13 +654,13 @@
         <v>15</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.974049900676195</v>
+        <v>-0.625430312013187</v>
       </c>
       <c r="G5" t="n">
-        <v>2.50457528570857</v>
+        <v>2.27268478607981</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0214285714285714</v>
+        <v>-0.703571428571428</v>
       </c>
       <c r="I5" t="n">
         <v>0.54228855721393</v>
@@ -669,13 +669,13 @@
         <v>0.54228855721393</v>
       </c>
       <c r="K5" t="n">
-        <v>0.233830845771144</v>
+        <v>0.507462686567164</v>
       </c>
       <c r="L5" t="n">
-        <v>-1.01227757899116</v>
+        <v>-0.857779083014129</v>
       </c>
       <c r="M5" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="6">
@@ -695,28 +695,28 @@
         <v>15</v>
       </c>
       <c r="F6" t="n">
-        <v>-1.99845049292821</v>
+        <v>-1.273489341928</v>
       </c>
       <c r="G6" t="n">
-        <v>54.2040744748085</v>
+        <v>47.1986909053332</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.77778277376493</v>
+        <v>-0.95341114203443</v>
       </c>
       <c r="I6" t="n">
-        <v>0.855721393034826</v>
+        <v>0.825870646766169</v>
       </c>
       <c r="J6" t="n">
-        <v>0.855721393034826</v>
+        <v>0.825870646766169</v>
       </c>
       <c r="K6" t="n">
-        <v>0.517412935323383</v>
+        <v>0.696517412935323</v>
       </c>
       <c r="L6" t="n">
-        <v>-1.11376584736152</v>
+        <v>-0.71784958006375</v>
       </c>
       <c r="M6" t="n">
-        <v>0.895522388059701</v>
+        <v>0.849466950959488</v>
       </c>
     </row>
     <row r="7">
@@ -736,28 +736,28 @@
         <v>14</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.487687452762323</v>
+        <v>-0.601226422449514</v>
       </c>
       <c r="G7" t="n">
-        <v>6.74168893752227</v>
+        <v>6.99421912084154</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.533040940639221</v>
+        <v>0.024255803055623</v>
       </c>
       <c r="I7" t="n">
-        <v>0.388059701492537</v>
+        <v>0.502487562189055</v>
       </c>
       <c r="J7" t="n">
-        <v>0.388059701492537</v>
+        <v>0.502487562189055</v>
       </c>
       <c r="K7" t="n">
-        <v>0.373134328358209</v>
+        <v>0.194029850746269</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.86553732032533</v>
+        <v>-0.72586792418767</v>
       </c>
       <c r="M7" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="8">
@@ -777,28 +777,28 @@
         <v>14</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.896261497646057</v>
+        <v>-0.608013749367726</v>
       </c>
       <c r="G8" t="n">
-        <v>11.8071046271769</v>
+        <v>10.8727443621744</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.969230769230769</v>
+        <v>-0.995604395604396</v>
       </c>
       <c r="I8" t="n">
-        <v>0.562189054726368</v>
+        <v>0.54726368159204</v>
       </c>
       <c r="J8" t="n">
-        <v>0.562189054726368</v>
+        <v>0.54726368159204</v>
       </c>
       <c r="K8" t="n">
-        <v>0.810945273631841</v>
+        <v>0.935323383084577</v>
       </c>
       <c r="L8" t="n">
-        <v>-1.58269160733885</v>
+        <v>-0.723163333052462</v>
       </c>
       <c r="M8" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="9">
@@ -818,28 +818,28 @@
         <v>14</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.184904729225614</v>
+        <v>-0.221870180006464</v>
       </c>
       <c r="G9" t="n">
-        <v>1590.32779135472</v>
+        <v>1614.94399127263</v>
       </c>
       <c r="H9" t="n">
-        <v>-0.986813186813187</v>
+        <v>-0.982417582417582</v>
       </c>
       <c r="I9" t="n">
-        <v>0.139303482587065</v>
+        <v>0.169154228855721</v>
       </c>
       <c r="J9" t="n">
-        <v>0.139303482587065</v>
+        <v>0.169154228855721</v>
       </c>
       <c r="K9" t="n">
-        <v>0.865671641791045</v>
+        <v>0.850746268656716</v>
       </c>
       <c r="L9" t="n">
-        <v>-1.74443268818879</v>
+        <v>-0.828557949836656</v>
       </c>
       <c r="M9" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="10">
@@ -859,28 +859,28 @@
         <v>14</v>
       </c>
       <c r="F10" t="n">
-        <v>-1.22188959304816</v>
+        <v>-0.947267850102067</v>
       </c>
       <c r="G10" t="n">
-        <v>2026.43988629061</v>
+        <v>1897.07864127603</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.885714285714286</v>
+        <v>-0.986813186813187</v>
       </c>
       <c r="I10" t="n">
-        <v>0.651741293532338</v>
+        <v>0.696517412935323</v>
       </c>
       <c r="J10" t="n">
-        <v>0.651741293532338</v>
+        <v>0.696517412935323</v>
       </c>
       <c r="K10" t="n">
-        <v>0.666666666666667</v>
+        <v>0.860696517412935</v>
       </c>
       <c r="L10" t="n">
-        <v>-1.69465881022022</v>
+        <v>-0.809725808901778</v>
       </c>
       <c r="M10" t="n">
-        <v>0.895522388059701</v>
+        <v>0.828358208955224</v>
       </c>
     </row>
     <row r="11">
@@ -900,28 +900,28 @@
         <v>14</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.178308365821654</v>
+        <v>-0.277703772717157</v>
       </c>
       <c r="G11" t="n">
-        <v>1.94012416794304</v>
+        <v>2.02029660337335</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.340659340659341</v>
+        <v>-0.217582417582418</v>
       </c>
       <c r="I11" t="n">
-        <v>0.109452736318408</v>
+        <v>0.288557213930348</v>
       </c>
       <c r="J11" t="n">
-        <v>0.109452736318408</v>
+        <v>0.288557213930348</v>
       </c>
       <c r="K11" t="n">
-        <v>0.313432835820896</v>
+        <v>0.26865671641791</v>
       </c>
       <c r="L11" t="n">
-        <v>-1.84837296896866</v>
+        <v>-0.705549022923467</v>
       </c>
       <c r="M11" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="12">
@@ -941,28 +941,28 @@
         <v>14</v>
       </c>
       <c r="F12" t="n">
-        <v>-1.46738015589463</v>
+        <v>-1.41390713244239</v>
       </c>
       <c r="G12" t="n">
-        <v>50.071175346186</v>
+        <v>49.525632549908</v>
       </c>
       <c r="H12" t="n">
-        <v>-0.902878556817261</v>
+        <v>-0.911708664952393</v>
       </c>
       <c r="I12" t="n">
-        <v>0.746268656716418</v>
+        <v>0.865671641791045</v>
       </c>
       <c r="J12" t="n">
-        <v>0.746268656716418</v>
+        <v>0.865671641791045</v>
       </c>
       <c r="K12" t="n">
-        <v>0.626865671641791</v>
+        <v>0.676616915422886</v>
       </c>
       <c r="L12" t="n">
-        <v>-1.53315946119574</v>
+        <v>-0.695061097811479</v>
       </c>
       <c r="M12" t="n">
-        <v>0.895522388059701</v>
+        <v>0.865671641791045</v>
       </c>
     </row>
     <row r="13">
@@ -982,28 +982,28 @@
         <v>13</v>
       </c>
       <c r="F13" t="n">
-        <v>-2.78600086795155</v>
+        <v>-0.390339669627938</v>
       </c>
       <c r="G13" t="n">
-        <v>11.150478222857</v>
+        <v>6.75715056995621</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.267218644822196</v>
+        <v>0.201102691464127</v>
       </c>
       <c r="I13" t="n">
-        <v>0.970149253731343</v>
+        <v>0.3681592039801</v>
       </c>
       <c r="J13" t="n">
-        <v>0.970149253731343</v>
+        <v>0.3681592039801</v>
       </c>
       <c r="K13" t="n">
-        <v>0.278606965174129</v>
+        <v>0.119402985074627</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.879535479482083</v>
+        <v>-0.717118807479813</v>
       </c>
       <c r="M13" t="n">
-        <v>0.970149253731343</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="14">
@@ -1023,28 +1023,28 @@
         <v>15</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.875424693947197</v>
+        <v>-0.59514445504856</v>
       </c>
       <c r="G14" t="n">
-        <v>11.4040539132123</v>
+        <v>10.5174257814494</v>
       </c>
       <c r="H14" t="n">
-        <v>0.00714285714285714</v>
+        <v>-0.621428571428571</v>
       </c>
       <c r="I14" t="n">
-        <v>0.696517412935323</v>
+        <v>0.557213930348259</v>
       </c>
       <c r="J14" t="n">
-        <v>0.696517412935323</v>
+        <v>0.557213930348259</v>
       </c>
       <c r="K14" t="n">
-        <v>0.228855721393035</v>
+        <v>0.447761194029851</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.81002907464454</v>
+        <v>-0.825831178406279</v>
       </c>
       <c r="M14" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="15">
@@ -1064,28 +1064,28 @@
         <v>15</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.903558805123857</v>
+        <v>-1.21215233829176</v>
       </c>
       <c r="G15" t="n">
-        <v>1947.89622813238</v>
+        <v>2099.85923855</v>
       </c>
       <c r="H15" t="n">
-        <v>-0.871428571428571</v>
+        <v>-0.925</v>
       </c>
       <c r="I15" t="n">
-        <v>0.805970149253731</v>
+        <v>0.81592039800995</v>
       </c>
       <c r="J15" t="n">
-        <v>0.805970149253731</v>
+        <v>0.81592039800995</v>
       </c>
       <c r="K15" t="n">
-        <v>0.6318407960199</v>
+        <v>0.661691542288557</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.697142312641595</v>
+        <v>-0.916709645618213</v>
       </c>
       <c r="M15" t="n">
-        <v>0.895522388059701</v>
+        <v>0.849466950959488</v>
       </c>
     </row>
     <row r="16">
@@ -1105,28 +1105,28 @@
         <v>15</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.328437237305923</v>
+        <v>-0.304669607149153</v>
       </c>
       <c r="G16" t="n">
-        <v>1513.77550441384</v>
+        <v>1500.17258835118</v>
       </c>
       <c r="H16" t="n">
         <v>-1</v>
       </c>
       <c r="I16" t="n">
-        <v>0.393034825870647</v>
+        <v>0.412935323383085</v>
       </c>
       <c r="J16" t="n">
-        <v>0.393034825870647</v>
+        <v>0.412935323383085</v>
       </c>
       <c r="K16" t="n">
         <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>-0.6709887991904</v>
+        <v>-0.810441510594059</v>
       </c>
       <c r="M16" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="17">
@@ -1146,28 +1146,28 @@
         <v>15</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.486602776823715</v>
+        <v>0.481548521760664</v>
       </c>
       <c r="G17" t="n">
-        <v>2.19487805795113</v>
+        <v>1.29618498302141</v>
       </c>
       <c r="H17" t="n">
-        <v>0.828571428571429</v>
+        <v>0.792857142857143</v>
       </c>
       <c r="I17" t="n">
-        <v>0.492537313432836</v>
+        <v>0.0248756218905473</v>
       </c>
       <c r="J17" t="n">
-        <v>0.492537313432836</v>
+        <v>0.0248756218905473</v>
       </c>
       <c r="K17" t="n">
-        <v>0.0199004975124378</v>
+        <v>0.0149253731343284</v>
       </c>
       <c r="L17" t="n">
-        <v>-0.796287683722316</v>
+        <v>-0.812815714754323</v>
       </c>
       <c r="M17" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="18">
@@ -1187,28 +1187,28 @@
         <v>15</v>
       </c>
       <c r="F18" t="n">
-        <v>-1.46602661866864</v>
+        <v>-0.755105088344304</v>
       </c>
       <c r="G18" t="n">
-        <v>48.8435149379277</v>
+        <v>41.2059178371211</v>
       </c>
       <c r="H18" t="n">
-        <v>-0.649333883017429</v>
+        <v>-0.959650904459459</v>
       </c>
       <c r="I18" t="n">
-        <v>0.870646766169154</v>
+        <v>0.676616915422886</v>
       </c>
       <c r="J18" t="n">
-        <v>0.870646766169154</v>
+        <v>0.676616915422886</v>
       </c>
       <c r="K18" t="n">
-        <v>0.432835820895522</v>
+        <v>0.746268656716418</v>
       </c>
       <c r="L18" t="n">
-        <v>-0.858213643828974</v>
+        <v>-0.909205048315741</v>
       </c>
       <c r="M18" t="n">
-        <v>0.895522388059701</v>
+        <v>0.828358208955224</v>
       </c>
     </row>
     <row r="19">
@@ -1228,28 +1228,28 @@
         <v>14</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.258415350377003</v>
+        <v>-0.22288604197574</v>
       </c>
       <c r="G19" t="n">
-        <v>7.41042649760461</v>
+        <v>7.30506684551492</v>
       </c>
       <c r="H19" t="n">
-        <v>-1</v>
+        <v>-0.995584988962472</v>
       </c>
       <c r="I19" t="n">
-        <v>0.298507462686567</v>
+        <v>0.293532338308458</v>
       </c>
       <c r="J19" t="n">
-        <v>0.298507462686567</v>
+        <v>0.293532338308458</v>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>0.840796019900497</v>
       </c>
       <c r="L19" t="n">
-        <v>-0.846459209176287</v>
+        <v>-0.571527601438834</v>
       </c>
       <c r="M19" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="20">
@@ -1269,28 +1269,28 @@
         <v>15</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.598465128354245</v>
+        <v>-0.597120044184857</v>
       </c>
       <c r="G20" t="n">
-        <v>10.8576306386392</v>
+        <v>10.8530614114242</v>
       </c>
       <c r="H20" t="n">
-        <v>-0.0607142857142857</v>
+        <v>0.0392857142857143</v>
       </c>
       <c r="I20" t="n">
-        <v>0.666666666666667</v>
+        <v>0.696517412935323</v>
       </c>
       <c r="J20" t="n">
-        <v>0.666666666666667</v>
+        <v>0.696517412935323</v>
       </c>
       <c r="K20" t="n">
-        <v>0.45273631840796</v>
+        <v>0.373134328358209</v>
       </c>
       <c r="L20" t="n">
-        <v>-0.472476138582422</v>
+        <v>-0.452946696479802</v>
       </c>
       <c r="M20" t="n">
-        <v>0.895522388059701</v>
+        <v>0.828358208955224</v>
       </c>
     </row>
     <row r="21">
@@ -1310,28 +1310,28 @@
         <v>15</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.714629731753571</v>
+        <v>-0.503741384609393</v>
       </c>
       <c r="G21" t="n">
-        <v>1864.0024534942</v>
+        <v>1745.61265075814</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.435714285714286</v>
+        <v>-0.232142857142857</v>
       </c>
       <c r="I21" t="n">
-        <v>0.666666666666667</v>
+        <v>0.552238805970149</v>
       </c>
       <c r="J21" t="n">
-        <v>0.666666666666667</v>
+        <v>0.552238805970149</v>
       </c>
       <c r="K21" t="n">
-        <v>0.805970149253731</v>
+        <v>0.611940298507463</v>
       </c>
       <c r="L21" t="n">
-        <v>-0.547734689118541</v>
+        <v>-0.533971414778284</v>
       </c>
       <c r="M21" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="22">
@@ -1351,28 +1351,28 @@
         <v>15</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.584084913895187</v>
+        <v>-0.380193050634186</v>
       </c>
       <c r="G22" t="n">
-        <v>1674.40705915574</v>
+        <v>1562.9379463826</v>
       </c>
       <c r="H22" t="n">
-        <v>-0.182142857142857</v>
+        <v>0.0178571428571429</v>
       </c>
       <c r="I22" t="n">
-        <v>0.557213930348259</v>
+        <v>0.398009950248756</v>
       </c>
       <c r="J22" t="n">
-        <v>0.557213930348259</v>
+        <v>0.398009950248756</v>
       </c>
       <c r="K22" t="n">
-        <v>0.567164179104478</v>
+        <v>0.358208955223881</v>
       </c>
       <c r="L22" t="n">
-        <v>-0.557543932861</v>
+        <v>-0.542580878901802</v>
       </c>
       <c r="M22" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="23">
@@ -1392,28 +1392,28 @@
         <v>15</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.275563350728128</v>
+        <v>-0.247743432546817</v>
       </c>
       <c r="G23" t="n">
-        <v>2.01328864346524</v>
+        <v>1.99121279270042</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.0535714285714286</v>
+        <v>-0.0607142857142857</v>
       </c>
       <c r="I23" t="n">
-        <v>0.358208955223881</v>
+        <v>0.343283582089552</v>
       </c>
       <c r="J23" t="n">
-        <v>0.358208955223881</v>
+        <v>0.343283582089552</v>
       </c>
       <c r="K23" t="n">
-        <v>0.512437810945274</v>
+        <v>0.522388059701492</v>
       </c>
       <c r="L23" t="n">
-        <v>-0.516679836846758</v>
+        <v>-0.517472620772991</v>
       </c>
       <c r="M23" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="24">
@@ -1433,28 +1433,28 @@
         <v>15</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.338453486826809</v>
+        <v>-0.210899468891642</v>
       </c>
       <c r="G24" t="n">
-        <v>36.2147201649462</v>
+        <v>34.44589999189</v>
       </c>
       <c r="H24" t="n">
-        <v>-0.0107527572409898</v>
+        <v>0.139785844132868</v>
       </c>
       <c r="I24" t="n">
-        <v>0.313432835820896</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="J24" t="n">
-        <v>0.313432835820896</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="K24" t="n">
-        <v>0.318407960199005</v>
+        <v>0.17910447761194</v>
       </c>
       <c r="L24" t="n">
-        <v>-0.600947510834579</v>
+        <v>-0.576088269598908</v>
       </c>
       <c r="M24" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="25">
@@ -1474,28 +1474,28 @@
         <v>14</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.262349049706547</v>
+        <v>-0.248873530960861</v>
       </c>
       <c r="G25" t="n">
-        <v>6.2101571300419</v>
+        <v>6.17692162258841</v>
       </c>
       <c r="H25" t="n">
-        <v>0.0308370792105334</v>
+        <v>0.0991191831767146</v>
       </c>
       <c r="I25" t="n">
-        <v>0.26865671641791</v>
+        <v>0.248756218905473</v>
       </c>
       <c r="J25" t="n">
-        <v>0.26865671641791</v>
+        <v>0.248756218905473</v>
       </c>
       <c r="K25" t="n">
-        <v>0.338308457711443</v>
+        <v>0.253731343283582</v>
       </c>
       <c r="L25" t="n">
-        <v>-0.644718723738239</v>
+        <v>-0.652551693292422</v>
       </c>
       <c r="M25" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="26">
@@ -1515,28 +1515,28 @@
         <v>14</v>
       </c>
       <c r="F26" t="n">
-        <v>-1.35871715366133</v>
+        <v>-0.8142114203871</v>
       </c>
       <c r="G26" t="n">
-        <v>13.1683763736421</v>
+        <v>11.5488368574811</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.70989010989011</v>
+        <v>-0.6</v>
       </c>
       <c r="I26" t="n">
-        <v>0.860696517412935</v>
+        <v>0.72636815920398</v>
       </c>
       <c r="J26" t="n">
-        <v>0.860696517412935</v>
+        <v>0.72636815920398</v>
       </c>
       <c r="K26" t="n">
-        <v>0.955223880597015</v>
+        <v>0.90547263681592</v>
       </c>
       <c r="L26" t="n">
-        <v>-0.66520091938375</v>
+        <v>-0.606530808016106</v>
       </c>
       <c r="M26" t="n">
-        <v>0.895522388059701</v>
+        <v>0.828358208955224</v>
       </c>
     </row>
     <row r="27">
@@ -1556,28 +1556,28 @@
         <v>14</v>
       </c>
       <c r="F27" t="n">
-        <v>-0.745896449248079</v>
+        <v>-0.565991674072742</v>
       </c>
       <c r="G27" t="n">
-        <v>1930.43050987003</v>
+        <v>1828.26715143658</v>
       </c>
       <c r="H27" t="n">
-        <v>-0.687912087912088</v>
+        <v>-0.657142857142857</v>
       </c>
       <c r="I27" t="n">
-        <v>0.616915422885572</v>
+        <v>0.54726368159204</v>
       </c>
       <c r="J27" t="n">
-        <v>0.616915422885572</v>
+        <v>0.54726368159204</v>
       </c>
       <c r="K27" t="n">
         <v>0.940298507462687</v>
       </c>
       <c r="L27" t="n">
-        <v>-0.654034169469455</v>
+        <v>-0.622798886862543</v>
       </c>
       <c r="M27" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="28">
@@ -1597,28 +1597,28 @@
         <v>14</v>
       </c>
       <c r="F28" t="n">
-        <v>-0.479131996945422</v>
+        <v>-0.269244016973327</v>
       </c>
       <c r="G28" t="n">
-        <v>1653.39246323245</v>
+        <v>1531.59891528459</v>
       </c>
       <c r="H28" t="n">
-        <v>-0.208791208791209</v>
+        <v>-0.191208791208791</v>
       </c>
       <c r="I28" t="n">
-        <v>0.427860696517413</v>
+        <v>0.278606965174129</v>
       </c>
       <c r="J28" t="n">
-        <v>0.427860696517413</v>
+        <v>0.278606965174129</v>
       </c>
       <c r="K28" t="n">
-        <v>0.587064676616915</v>
+        <v>0.572139303482587</v>
       </c>
       <c r="L28" t="n">
-        <v>-0.697020350522995</v>
+        <v>-0.652858128822046</v>
       </c>
       <c r="M28" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="29">
@@ -1638,28 +1638,28 @@
         <v>14</v>
       </c>
       <c r="F29" t="n">
-        <v>-0.237730008398054</v>
+        <v>-0.322358674942473</v>
       </c>
       <c r="G29" t="n">
-        <v>1.9884423550693</v>
+        <v>2.05529743110891</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0549450549450549</v>
+        <v>-0.235164835164835</v>
       </c>
       <c r="I29" t="n">
-        <v>0.189054726368159</v>
+        <v>0.328358208955224</v>
       </c>
       <c r="J29" t="n">
-        <v>0.189054726368159</v>
+        <v>0.328358208955224</v>
       </c>
       <c r="K29" t="n">
-        <v>0.26865671641791</v>
+        <v>0.601990049751244</v>
       </c>
       <c r="L29" t="n">
-        <v>-0.686416156557</v>
+        <v>-0.638447911144065</v>
       </c>
       <c r="M29" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="30">
@@ -1679,28 +1679,28 @@
         <v>14</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.837878802783345</v>
+        <v>-0.75860312322287</v>
       </c>
       <c r="G30" t="n">
-        <v>43.2143700545766</v>
+        <v>42.2720852922781</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.29801614956071</v>
+        <v>-0.183224743803992</v>
       </c>
       <c r="I30" t="n">
-        <v>0.721393034825871</v>
+        <v>0.736318407960199</v>
       </c>
       <c r="J30" t="n">
-        <v>0.721393034825871</v>
+        <v>0.736318407960199</v>
       </c>
       <c r="K30" t="n">
-        <v>0.661691542288557</v>
+        <v>0.557213930348259</v>
       </c>
       <c r="L30" t="n">
-        <v>-0.599438879282538</v>
+        <v>-0.564232275553215</v>
       </c>
       <c r="M30" t="n">
-        <v>0.895522388059701</v>
+        <v>0.828358208955224</v>
       </c>
     </row>
     <row r="31">
@@ -1720,28 +1720,28 @@
         <v>13</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.403555304747535</v>
+        <v>-0.246464638433984</v>
       </c>
       <c r="G31" t="n">
-        <v>6.78918908341402</v>
+        <v>6.39798356885888</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.066115953358069</v>
+        <v>0.126722243936299</v>
       </c>
       <c r="I31" t="n">
-        <v>0.358208955223881</v>
+        <v>0.278606965174129</v>
       </c>
       <c r="J31" t="n">
-        <v>0.358208955223881</v>
+        <v>0.278606965174129</v>
       </c>
       <c r="K31" t="n">
-        <v>0.437810945273632</v>
+        <v>0.278606965174129</v>
       </c>
       <c r="L31" t="n">
-        <v>-0.734427875443146</v>
+        <v>-0.685683097489931</v>
       </c>
       <c r="M31" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="32">
@@ -1761,28 +1761,28 @@
         <v>15</v>
       </c>
       <c r="F32" t="n">
-        <v>-0.508686257464333</v>
+        <v>-0.293305294861217</v>
       </c>
       <c r="G32" t="n">
-        <v>10.2284285064938</v>
+        <v>9.47021795982088</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.0714285714285714</v>
+        <v>0.1</v>
       </c>
       <c r="I32" t="n">
-        <v>0.557213930348259</v>
+        <v>0.328358208955224</v>
       </c>
       <c r="J32" t="n">
-        <v>0.557213930348259</v>
+        <v>0.328358208955224</v>
       </c>
       <c r="K32" t="n">
-        <v>0.412935323383085</v>
+        <v>0.26865671641791</v>
       </c>
       <c r="L32" t="n">
-        <v>-0.527079059536174</v>
+        <v>-0.539240295760514</v>
       </c>
       <c r="M32" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="33">
@@ -1802,28 +1802,28 @@
         <v>15</v>
       </c>
       <c r="F33" t="n">
-        <v>-0.676083771307747</v>
+        <v>-0.546299962475635</v>
       </c>
       <c r="G33" t="n">
-        <v>1827.80780847301</v>
+        <v>1755.61604159832</v>
       </c>
       <c r="H33" t="n">
-        <v>-0.364285714285714</v>
+        <v>-0.267857142857143</v>
       </c>
       <c r="I33" t="n">
-        <v>0.701492537313433</v>
+        <v>0.567164179104478</v>
       </c>
       <c r="J33" t="n">
-        <v>0.701492537313433</v>
+        <v>0.567164179104478</v>
       </c>
       <c r="K33" t="n">
-        <v>0.721393034825871</v>
+        <v>0.606965174129353</v>
       </c>
       <c r="L33" t="n">
-        <v>-0.523416676068986</v>
+        <v>-0.548868960802837</v>
       </c>
       <c r="M33" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="34">
@@ -1843,28 +1843,28 @@
         <v>15</v>
       </c>
       <c r="F34" t="n">
-        <v>-0.374302403721699</v>
+        <v>-0.36025070046376</v>
       </c>
       <c r="G34" t="n">
-        <v>1539.68580540137</v>
+        <v>1531.79423968262</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.239285714285714</v>
+        <v>-0.217857142857143</v>
       </c>
       <c r="I34" t="n">
-        <v>0.45273631840796</v>
+        <v>0.422885572139304</v>
       </c>
       <c r="J34" t="n">
-        <v>0.45273631840796</v>
+        <v>0.422885572139304</v>
       </c>
       <c r="K34" t="n">
-        <v>0.54726368159204</v>
+        <v>0.562189054726368</v>
       </c>
       <c r="L34" t="n">
-        <v>-0.5224559717256</v>
+        <v>-0.544327821823764</v>
       </c>
       <c r="M34" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="35">
@@ -1884,28 +1884,28 @@
         <v>15</v>
       </c>
       <c r="F35" t="n">
-        <v>-0.461967409321836</v>
+        <v>-0.258309465394461</v>
       </c>
       <c r="G35" t="n">
-        <v>2.17661577660218</v>
+        <v>2.01932703091343</v>
       </c>
       <c r="H35" t="n">
-        <v>-0.153571428571429</v>
+        <v>0.189285714285714</v>
       </c>
       <c r="I35" t="n">
-        <v>0.54726368159204</v>
+        <v>0.303482587064677</v>
       </c>
       <c r="J35" t="n">
-        <v>0.54726368159204</v>
+        <v>0.303482587064677</v>
       </c>
       <c r="K35" t="n">
-        <v>0.517412935323383</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="L35" t="n">
-        <v>-0.470481529642712</v>
+        <v>-0.484647601294485</v>
       </c>
       <c r="M35" t="n">
-        <v>0.895522388059701</v>
+        <v>0.785304247990815</v>
       </c>
     </row>
     <row r="36">
@@ -1925,28 +1925,28 @@
         <v>15</v>
       </c>
       <c r="F36" t="n">
-        <v>-0.944469729484661</v>
+        <v>-0.812121916309217</v>
       </c>
       <c r="G36" t="n">
-        <v>43.3719174897986</v>
+        <v>41.86988191067</v>
       </c>
       <c r="H36" t="n">
-        <v>-0.129149280600152</v>
+        <v>-0.256504821191968</v>
       </c>
       <c r="I36" t="n">
-        <v>0.850746268656716</v>
+        <v>0.791044776119403</v>
       </c>
       <c r="J36" t="n">
-        <v>0.850746268656716</v>
+        <v>0.791044776119403</v>
       </c>
       <c r="K36" t="n">
-        <v>0.477611940298507</v>
+        <v>0.671641791044776</v>
       </c>
       <c r="L36" t="n">
-        <v>-0.524305798078358</v>
+        <v>-0.51431422242233</v>
       </c>
       <c r="M36" t="n">
-        <v>0.895522388059701</v>
+        <v>0.849466950959488</v>
       </c>
     </row>
     <row r="37">
@@ -1966,28 +1966,28 @@
         <v>14</v>
       </c>
       <c r="F37" t="n">
-        <v>-0.545047067906229</v>
+        <v>-0.569367123723489</v>
       </c>
       <c r="G37" t="n">
-        <v>8.21111354022207</v>
+        <v>8.27548537611177</v>
       </c>
       <c r="H37" t="n">
-        <v>-0.306168143590296</v>
+        <v>-0.30176284656022</v>
       </c>
       <c r="I37" t="n">
-        <v>0.611940298507463</v>
+        <v>0.601990049751244</v>
       </c>
       <c r="J37" t="n">
-        <v>0.611940298507463</v>
+        <v>0.601990049751244</v>
       </c>
       <c r="K37" t="n">
-        <v>0.651741293532338</v>
+        <v>0.646766169154229</v>
       </c>
       <c r="L37" t="n">
-        <v>-0.529082011182215</v>
+        <v>-0.534397443297713</v>
       </c>
       <c r="M37" t="n">
-        <v>0.895522388059701</v>
+        <v>0.802653399668325</v>
       </c>
     </row>
   </sheetData>
@@ -2044,7 +2044,7 @@
         <v>9.43</v>
       </c>
       <c r="G2" t="n">
-        <v>0.295297964331835</v>
+        <v>-3.59225753979196</v>
       </c>
     </row>
     <row r="3">
@@ -2090,7 +2090,7 @@
         <v>13.69</v>
       </c>
       <c r="G4" t="n">
-        <v>-7.4947658036656</v>
+        <v>4.63785714285714</v>
       </c>
     </row>
     <row r="5">
@@ -2113,7 +2113,7 @@
         <v>10.45</v>
       </c>
       <c r="G5" t="n">
-        <v>5.36046747044403</v>
+        <v>4.86928571428571</v>
       </c>
     </row>
     <row r="6">
@@ -2136,7 +2136,7 @@
         <v>14.93</v>
       </c>
       <c r="G6" t="n">
-        <v>4.9150605726497</v>
+        <v>4.54928571428571</v>
       </c>
     </row>
     <row r="7">
@@ -2159,7 +2159,7 @@
         <v>13.79</v>
       </c>
       <c r="G7" t="n">
-        <v>-24.8162331077139</v>
+        <v>4.63071428571429</v>
       </c>
     </row>
     <row r="8">
@@ -2205,7 +2205,7 @@
         <v>0.79</v>
       </c>
       <c r="G9" t="n">
-        <v>9.08065510429014</v>
+        <v>5.55928571428571</v>
       </c>
     </row>
     <row r="10">
@@ -2228,7 +2228,7 @@
         <v>0.85</v>
       </c>
       <c r="G10" t="n">
-        <v>3.62503521301866</v>
+        <v>5.555</v>
       </c>
     </row>
     <row r="11">
@@ -2251,7 +2251,7 @@
         <v>-4.09</v>
       </c>
       <c r="G11" t="n">
-        <v>5.87077128053465</v>
+        <v>5.90785714285714</v>
       </c>
     </row>
     <row r="12">
@@ -2274,7 +2274,7 @@
         <v>-0.74</v>
       </c>
       <c r="G12" t="n">
-        <v>3.75360795285026</v>
+        <v>5.66857142857143</v>
       </c>
     </row>
     <row r="13">
@@ -2297,7 +2297,7 @@
         <v>-1.86</v>
       </c>
       <c r="G13" t="n">
-        <v>6.50331475881258</v>
+        <v>5.74857142857143</v>
       </c>
     </row>
     <row r="14">
@@ -2343,7 +2343,7 @@
         <v>-5.99</v>
       </c>
       <c r="G15" t="n">
-        <v>6.57961132928214</v>
+        <v>6.04357142857143</v>
       </c>
     </row>
     <row r="16">
@@ -2366,7 +2366,7 @@
         <v>-0.48</v>
       </c>
       <c r="G16" t="n">
-        <v>3.97353020321495</v>
+        <v>5.65</v>
       </c>
     </row>
     <row r="17">
@@ -2389,7 +2389,7 @@
         <v>874.31</v>
       </c>
       <c r="G17" t="n">
-        <v>-229.962857142857</v>
+        <v>-1408.99857406496</v>
       </c>
     </row>
     <row r="18">
@@ -2642,7 +2642,7 @@
         <v>-2646.36</v>
       </c>
       <c r="G28" t="n">
-        <v>21.5135714285715</v>
+        <v>30.3583272211975</v>
       </c>
     </row>
     <row r="29">
@@ -2734,7 +2734,7 @@
         <v>517.34</v>
       </c>
       <c r="G32" t="n">
-        <v>58.8892857142856</v>
+        <v>-787.116938110589</v>
       </c>
     </row>
     <row r="33">
@@ -2780,7 +2780,7 @@
         <v>2790.83</v>
       </c>
       <c r="G34" t="n">
-        <v>-2419.60121215346</v>
+        <v>-103.502857142857</v>
       </c>
     </row>
     <row r="35">
@@ -2895,7 +2895,7 @@
         <v>-171.76</v>
       </c>
       <c r="G39" t="n">
-        <v>108.110714285714</v>
+        <v>481.950013018944</v>
       </c>
     </row>
     <row r="40">
@@ -2941,7 +2941,7 @@
         <v>-1503.6</v>
       </c>
       <c r="G41" t="n">
-        <v>203.242142857143</v>
+        <v>494.133601898367</v>
       </c>
     </row>
     <row r="42">
@@ -2987,7 +2987,7 @@
         <v>-2305.05</v>
       </c>
       <c r="G43" t="n">
-        <v>260.488571428571</v>
+        <v>276.046773529055</v>
       </c>
     </row>
     <row r="44">
@@ -3079,7 +3079,7 @@
         <v>1.706</v>
       </c>
       <c r="G47" t="n">
-        <v>3.50869609878778</v>
+        <v>-0.479857189444632</v>
       </c>
     </row>
     <row r="48">
@@ -3102,7 +3102,7 @@
         <v>4.218</v>
       </c>
       <c r="G48" t="n">
-        <v>1.941334630595</v>
+        <v>1.20951678605622</v>
       </c>
     </row>
     <row r="49">
@@ -3125,7 +3125,7 @@
         <v>1.578</v>
       </c>
       <c r="G49" t="n">
-        <v>4.0116752274803</v>
+        <v>3.82625470311401</v>
       </c>
     </row>
     <row r="50">
@@ -3148,7 +3148,7 @@
         <v>3.683</v>
       </c>
       <c r="G50" t="n">
-        <v>2.54842837353549</v>
+        <v>1.8335</v>
       </c>
     </row>
     <row r="51">
@@ -3171,7 +3171,7 @@
         <v>2.983</v>
       </c>
       <c r="G51" t="n">
-        <v>1.68732356884428</v>
+        <v>0.29486090689584</v>
       </c>
     </row>
     <row r="52">
@@ -3194,7 +3194,7 @@
         <v>2.44</v>
       </c>
       <c r="G52" t="n">
-        <v>5.22932714150403</v>
+        <v>1.92228571428571</v>
       </c>
     </row>
     <row r="53">
@@ -3217,7 +3217,7 @@
         <v>3.614</v>
       </c>
       <c r="G53" t="n">
-        <v>2.34681654552371</v>
+        <v>1.58867200574382</v>
       </c>
     </row>
     <row r="54">
@@ -3240,7 +3240,7 @@
         <v>0.579999999999998</v>
       </c>
       <c r="G54" t="n">
-        <v>2.88568233061863</v>
+        <v>2.24349489163752</v>
       </c>
     </row>
     <row r="55">
@@ -3263,7 +3263,7 @@
         <v>-1.918</v>
       </c>
       <c r="G55" t="n">
-        <v>2.23357142857143</v>
+        <v>2.22309232050584</v>
       </c>
     </row>
     <row r="56">
@@ -3286,7 +3286,7 @@
         <v>0.672000000000001</v>
       </c>
       <c r="G56" t="n">
-        <v>-0.305663328667519</v>
+        <v>2.04857142857143</v>
       </c>
     </row>
     <row r="57">
@@ -3309,7 +3309,7 @@
         <v>0.352999999999998</v>
       </c>
       <c r="G57" t="n">
-        <v>0.525517266068184</v>
+        <v>2.07135714285714</v>
       </c>
     </row>
     <row r="58">
@@ -3332,7 +3332,7 @@
         <v>5.08900000000001</v>
       </c>
       <c r="G58" t="n">
-        <v>1.97489445864848</v>
+        <v>1.83054109183315</v>
       </c>
     </row>
     <row r="59">
@@ -3355,7 +3355,7 @@
         <v>0.181000000000001</v>
       </c>
       <c r="G59" t="n">
-        <v>2.15768994333134</v>
+        <v>2.45419958406174</v>
       </c>
     </row>
     <row r="60">
@@ -3378,7 +3378,7 @@
         <v>1.311</v>
       </c>
       <c r="G60" t="n">
-        <v>-0.947095759295908</v>
+        <v>2.21468319650986</v>
       </c>
     </row>
     <row r="61">
@@ -3401,7 +3401,7 @@
         <v>2.862</v>
       </c>
       <c r="G61" t="n">
-        <v>-2.15241719894983</v>
+        <v>1.37507996604291</v>
       </c>
     </row>
     <row r="62">
@@ -3470,7 +3470,7 @@
         <v>90</v>
       </c>
       <c r="G64" t="n">
-        <v>19.7076744158845</v>
+        <v>-3.85761982395725</v>
       </c>
     </row>
     <row r="65">
@@ -3516,7 +3516,7 @@
         <v>5</v>
       </c>
       <c r="G66" t="n">
-        <v>47.7732274026498</v>
+        <v>47.3552507013026</v>
       </c>
     </row>
     <row r="67">
@@ -3562,7 +3562,7 @@
         <v>65</v>
       </c>
       <c r="G68" t="n">
-        <v>146.539777226992</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="69">
@@ -3631,7 +3631,7 @@
         <v>5</v>
       </c>
       <c r="G71" t="n">
-        <v>140.12451123781</v>
+        <v>62.3860499127668</v>
       </c>
     </row>
     <row r="72">
@@ -3700,7 +3700,7 @@
         <v>18</v>
       </c>
       <c r="G74" t="n">
-        <v>45.8571428571428</v>
+        <v>48.1415211349746</v>
       </c>
     </row>
     <row r="75">
@@ -3723,7 +3723,7 @@
         <v>5</v>
       </c>
       <c r="G75" t="n">
-        <v>50.2945141673853</v>
+        <v>100.97390464627</v>
       </c>
     </row>
     <row r="76">
@@ -3746,7 +3746,7 @@
         <v>89</v>
       </c>
       <c r="G76" t="n">
-        <v>26.0151910496353</v>
+        <v>31.59774434814</v>
       </c>
     </row>
     <row r="77">
@@ -3769,7 +3769,7 @@
         <v>5</v>
       </c>
       <c r="G77" t="n">
-        <v>9.15384615384616</v>
+        <v>3.90511013531552</v>
       </c>
     </row>
     <row r="78">
@@ -3792,7 +3792,7 @@
         <v>14</v>
       </c>
       <c r="G78" t="n">
-        <v>8.42738647682263</v>
+        <v>9.31390702304854</v>
       </c>
     </row>
     <row r="79">
@@ -3815,7 +3815,7 @@
         <v>4</v>
       </c>
       <c r="G79" t="n">
-        <v>12.3673087655893</v>
+        <v>10.8071449210542</v>
       </c>
     </row>
     <row r="80">
@@ -3838,7 +3838,7 @@
         <v>11</v>
       </c>
       <c r="G80" t="n">
-        <v>9.44104796174055</v>
+        <v>10.952778735522</v>
       </c>
     </row>
     <row r="81">
@@ -3861,7 +3861,7 @@
         <v>10</v>
       </c>
       <c r="G81" t="n">
-        <v>9.59474531802724</v>
+        <v>11.5255249873369</v>
       </c>
     </row>
     <row r="82">
@@ -3884,7 +3884,7 @@
         <v>8</v>
       </c>
       <c r="G82" t="n">
-        <v>15.2536665084177</v>
+        <v>13.8893715743681</v>
       </c>
     </row>
     <row r="83">
@@ -3907,7 +3907,7 @@
         <v>6</v>
       </c>
       <c r="G83" t="n">
-        <v>9.65661975259776</v>
+        <v>8.1672867612092</v>
       </c>
     </row>
     <row r="84">
@@ -3930,7 +3930,7 @@
         <v>20</v>
       </c>
       <c r="G84" t="n">
-        <v>8.03351581098684</v>
+        <v>9.68433763878012</v>
       </c>
     </row>
     <row r="85">
@@ -3953,7 +3953,7 @@
         <v>7</v>
       </c>
       <c r="G85" t="n">
-        <v>9.32531650806795</v>
+        <v>9.36421122656187</v>
       </c>
     </row>
     <row r="86">
@@ -3976,7 +3976,7 @@
         <v>6</v>
       </c>
       <c r="G86" t="n">
-        <v>12.2437854876601</v>
+        <v>17.9944317017506</v>
       </c>
     </row>
     <row r="87">
@@ -3999,7 +3999,7 @@
         <v>16</v>
       </c>
       <c r="G87" t="n">
-        <v>8.71531169213263</v>
+        <v>9.78938086239785</v>
       </c>
     </row>
     <row r="88">
@@ -4045,7 +4045,7 @@
         <v>15</v>
       </c>
       <c r="G89" t="n">
-        <v>6.37379704342163</v>
+        <v>3.33703195082431</v>
       </c>
     </row>
     <row r="90">
@@ -4068,7 +4068,7 @@
         <v>1</v>
       </c>
       <c r="G90" t="n">
-        <v>8.92081813958406</v>
+        <v>9.46153846153846</v>
       </c>
     </row>
     <row r="91">
@@ -4114,7 +4114,7 @@
         <v>20.73</v>
       </c>
       <c r="G92" t="n">
-        <v>3.39769230769231</v>
+        <v>-3.12263992157248</v>
       </c>
     </row>
     <row r="93">
@@ -4137,7 +4137,7 @@
         <v>13.69</v>
       </c>
       <c r="G93" t="n">
-        <v>-14.7700815069756</v>
+        <v>3.93923076923077</v>
       </c>
     </row>
     <row r="94">
@@ -4367,7 +4367,7 @@
         <v>-5.99</v>
       </c>
       <c r="G103" t="n">
-        <v>7.20388568722972</v>
+        <v>12.0033799233388</v>
       </c>
     </row>
     <row r="104">
@@ -4413,7 +4413,7 @@
         <v>874.31</v>
       </c>
       <c r="G105" t="n">
-        <v>-288.866153846154</v>
+        <v>-323.078032536791</v>
       </c>
     </row>
     <row r="106">
@@ -4459,7 +4459,7 @@
         <v>1924.77</v>
       </c>
       <c r="G107" t="n">
-        <v>-369.670769230769</v>
+        <v>-707.269835717247</v>
       </c>
     </row>
     <row r="108">
@@ -4482,7 +4482,7 @@
         <v>274.62</v>
       </c>
       <c r="G108" t="n">
-        <v>-242.736153846154</v>
+        <v>-229.477028242272</v>
       </c>
     </row>
     <row r="109">
@@ -4528,7 +4528,7 @@
         <v>1276.8</v>
       </c>
       <c r="G110" t="n">
-        <v>-539.929909537273</v>
+        <v>-319.826923076923</v>
       </c>
     </row>
     <row r="111">
@@ -4551,7 +4551,7 @@
         <v>171.549999999999</v>
       </c>
       <c r="G111" t="n">
-        <v>-234.807692307692</v>
+        <v>-217.27462756719</v>
       </c>
     </row>
     <row r="112">
@@ -4666,7 +4666,7 @@
         <v>-1385.12</v>
       </c>
       <c r="G116" t="n">
-        <v>-115.063846153846</v>
+        <v>-111.114096593328</v>
       </c>
     </row>
     <row r="117">
@@ -4712,7 +4712,7 @@
         <v>-1268.92</v>
       </c>
       <c r="G118" t="n">
-        <v>-124.002307692308</v>
+        <v>-68.8151416531206</v>
       </c>
     </row>
     <row r="119">
@@ -4735,7 +4735,7 @@
         <v>517.34</v>
       </c>
       <c r="G119" t="n">
-        <v>-219.692245877041</v>
+        <v>-4.45538461538465</v>
       </c>
     </row>
     <row r="120">
@@ -4781,7 +4781,7 @@
         <v>2790.83</v>
       </c>
       <c r="G121" t="n">
-        <v>-179.339230769231</v>
+        <v>-507.673957224189</v>
       </c>
     </row>
     <row r="122">
@@ -4988,7 +4988,7 @@
         <v>-1179.58</v>
       </c>
       <c r="G130" t="n">
-        <v>161.168775561776</v>
+        <v>126.076923076923</v>
       </c>
     </row>
     <row r="131">
@@ -5011,7 +5011,7 @@
         <v>-1491.94</v>
       </c>
       <c r="G131" t="n">
-        <v>3968.33010894525</v>
+        <v>3092.20905634414</v>
       </c>
     </row>
     <row r="132">
@@ -5057,7 +5057,7 @@
         <v>1.706</v>
       </c>
       <c r="G133" t="n">
-        <v>1.97197599670164</v>
+        <v>2.54917206474958</v>
       </c>
     </row>
     <row r="134">
@@ -5080,7 +5080,7 @@
         <v>4.218</v>
       </c>
       <c r="G134" t="n">
-        <v>1.17406757961213</v>
+        <v>1.46722906935222</v>
       </c>
     </row>
     <row r="135">
@@ -5103,7 +5103,7 @@
         <v>1.578</v>
       </c>
       <c r="G135" t="n">
-        <v>0.799025422170216</v>
+        <v>0.52108318837091</v>
       </c>
     </row>
     <row r="136">
@@ -5126,7 +5126,7 @@
         <v>3.683</v>
       </c>
       <c r="G136" t="n">
-        <v>1.76050695914428</v>
+        <v>1.823534022233</v>
       </c>
     </row>
     <row r="137">
@@ -5149,7 +5149,7 @@
         <v>2.983</v>
       </c>
       <c r="G137" t="n">
-        <v>1.32629065483514</v>
+        <v>1.59330452753923</v>
       </c>
     </row>
     <row r="138">
@@ -5172,7 +5172,7 @@
         <v>2.44</v>
       </c>
       <c r="G138" t="n">
-        <v>1.9408710253894</v>
+        <v>2.05156425863351</v>
       </c>
     </row>
     <row r="139">
@@ -5195,7 +5195,7 @@
         <v>0.579999999999998</v>
       </c>
       <c r="G139" t="n">
-        <v>1.93523076923077</v>
+        <v>1.52644823002095</v>
       </c>
     </row>
     <row r="140">
@@ -5218,7 +5218,7 @@
         <v>-1.918</v>
       </c>
       <c r="G140" t="n">
-        <v>1.86327076870047</v>
+        <v>2.79003559532209</v>
       </c>
     </row>
     <row r="141">
@@ -5241,7 +5241,7 @@
         <v>0.672000000000001</v>
       </c>
       <c r="G141" t="n">
-        <v>1.92815384615385</v>
+        <v>1.7675983771508</v>
       </c>
     </row>
     <row r="142">
@@ -5264,7 +5264,7 @@
         <v>0.352999999999998</v>
       </c>
       <c r="G142" t="n">
-        <v>1.890547083809</v>
+        <v>1.96852647919441</v>
       </c>
     </row>
     <row r="143">
@@ -5310,7 +5310,7 @@
         <v>0.181000000000001</v>
       </c>
       <c r="G144" t="n">
-        <v>1.72962233703001</v>
+        <v>1.70011892506146</v>
       </c>
     </row>
     <row r="145">
@@ -5333,7 +5333,7 @@
         <v>1.311</v>
       </c>
       <c r="G145" t="n">
-        <v>1.91003984994611</v>
+        <v>1.43727584332503</v>
       </c>
     </row>
     <row r="146">
@@ -5356,7 +5356,7 @@
         <v>2.862</v>
       </c>
       <c r="G146" t="n">
-        <v>1.87394119846304</v>
+        <v>1.99121094505456</v>
       </c>
     </row>
     <row r="147">
@@ -5379,7 +5379,7 @@
         <v>54</v>
       </c>
       <c r="G147" t="n">
-        <v>36.4427620367146</v>
+        <v>34.9574906749181</v>
       </c>
     </row>
     <row r="148">
@@ -5471,7 +5471,7 @@
         <v>5</v>
       </c>
       <c r="G151" t="n">
-        <v>46.9940236210402</v>
+        <v>45.3846153846154</v>
       </c>
     </row>
     <row r="152">
@@ -5563,7 +5563,7 @@
         <v>5</v>
       </c>
       <c r="G155" t="n">
-        <v>72.021799482797</v>
+        <v>77.9557142609992</v>
       </c>
     </row>
     <row r="156">
@@ -5655,7 +5655,7 @@
         <v>5</v>
       </c>
       <c r="G159" t="n">
-        <v>135.705613256456</v>
+        <v>129.783342269034</v>
       </c>
     </row>
     <row r="160">
@@ -5701,7 +5701,7 @@
         <v>5</v>
       </c>
       <c r="G161" t="n">
-        <v>-27.5254410859815</v>
+        <v>-1.64892304076396</v>
       </c>
     </row>
     <row r="162">
@@ -5724,7 +5724,7 @@
         <v>14</v>
       </c>
       <c r="G162" t="n">
-        <v>8.5</v>
+        <v>11.6619267048792</v>
       </c>
     </row>
     <row r="163">
@@ -5747,7 +5747,7 @@
         <v>4</v>
       </c>
       <c r="G163" t="n">
-        <v>10.4194471165267</v>
+        <v>10.9135746225567</v>
       </c>
     </row>
     <row r="164">
@@ -5770,7 +5770,7 @@
         <v>11</v>
       </c>
       <c r="G164" t="n">
-        <v>14.10178173947</v>
+        <v>15.6752350787855</v>
       </c>
     </row>
     <row r="165">
@@ -5793,7 +5793,7 @@
         <v>10</v>
       </c>
       <c r="G165" t="n">
-        <v>8.53504847299982</v>
+        <v>6.79537581196603</v>
       </c>
     </row>
     <row r="166">
@@ -5816,7 +5816,7 @@
         <v>6</v>
       </c>
       <c r="G166" t="n">
-        <v>3.93161656556247</v>
+        <v>6.11098676514089</v>
       </c>
     </row>
     <row r="167">
@@ -5839,7 +5839,7 @@
         <v>20</v>
       </c>
       <c r="G167" t="n">
-        <v>8</v>
+        <v>9.41550917484378</v>
       </c>
     </row>
     <row r="168">
@@ -5862,7 +5862,7 @@
         <v>7</v>
       </c>
       <c r="G168" t="n">
-        <v>9.91079924905198</v>
+        <v>9.91834763480099</v>
       </c>
     </row>
     <row r="169">
@@ -5885,7 +5885,7 @@
         <v>6</v>
       </c>
       <c r="G169" t="n">
-        <v>11.7258345744703</v>
+        <v>10.9056315420365</v>
       </c>
     </row>
     <row r="170">
@@ -5908,7 +5908,7 @@
         <v>16</v>
       </c>
       <c r="G170" t="n">
-        <v>6.99713851775612</v>
+        <v>7.70360565443946</v>
       </c>
     </row>
     <row r="171">
@@ -5931,7 +5931,7 @@
         <v>1</v>
       </c>
       <c r="G171" t="n">
-        <v>9.04848812445999</v>
+        <v>7.6866145310432</v>
       </c>
     </row>
     <row r="172">
@@ -5954,7 +5954,7 @@
         <v>15</v>
       </c>
       <c r="G172" t="n">
-        <v>5.92295070901387</v>
+        <v>1.76892357241744</v>
       </c>
     </row>
     <row r="173">
@@ -5977,7 +5977,7 @@
         <v>1</v>
       </c>
       <c r="G173" t="n">
-        <v>8.57903318772484</v>
+        <v>6.54439156358514</v>
       </c>
     </row>
     <row r="174">
@@ -6000,7 +6000,7 @@
         <v>9.43</v>
       </c>
       <c r="G174" t="n">
-        <v>7.58279298935965</v>
+        <v>7.05191852392312</v>
       </c>
     </row>
     <row r="175">
@@ -6023,7 +6023,7 @@
         <v>20.73</v>
       </c>
       <c r="G175" t="n">
-        <v>3.3955698707418</v>
+        <v>0.582877753326255</v>
       </c>
     </row>
     <row r="176">
@@ -6046,7 +6046,7 @@
         <v>13.69</v>
       </c>
       <c r="G176" t="n">
-        <v>2.9043564933274</v>
+        <v>2.79651142521721</v>
       </c>
     </row>
     <row r="177">
@@ -6069,7 +6069,7 @@
         <v>10.45</v>
       </c>
       <c r="G177" t="n">
-        <v>4.35200178307523</v>
+        <v>4.10506324976776</v>
       </c>
     </row>
     <row r="178">
@@ -6092,7 +6092,7 @@
         <v>14.93</v>
       </c>
       <c r="G178" t="n">
-        <v>33.1148415580579</v>
+        <v>4.145</v>
       </c>
     </row>
     <row r="179">
@@ -6115,7 +6115,7 @@
         <v>13.79</v>
       </c>
       <c r="G179" t="n">
-        <v>3.21275570375928</v>
+        <v>3.11159617019263</v>
       </c>
     </row>
     <row r="180">
@@ -6138,7 +6138,7 @@
         <v>8.06</v>
       </c>
       <c r="G180" t="n">
-        <v>-16.05760463464</v>
+        <v>0.219118163031496</v>
       </c>
     </row>
     <row r="181">
@@ -6161,7 +6161,7 @@
         <v>0.79</v>
       </c>
       <c r="G181" t="n">
-        <v>5.10977343807979</v>
+        <v>4.55604118552488</v>
       </c>
     </row>
     <row r="182">
@@ -6184,7 +6184,7 @@
         <v>0.85</v>
       </c>
       <c r="G182" t="n">
-        <v>3.04615893821177</v>
+        <v>3.18480234774414</v>
       </c>
     </row>
     <row r="183">
@@ -6207,7 +6207,7 @@
         <v>-4.09</v>
       </c>
       <c r="G183" t="n">
-        <v>5.69011397604316</v>
+        <v>10.3728278494341</v>
       </c>
     </row>
     <row r="184">
@@ -6230,7 +6230,7 @@
         <v>-0.74</v>
       </c>
       <c r="G184" t="n">
-        <v>3.26407812673038</v>
+        <v>4.65303450716843</v>
       </c>
     </row>
     <row r="185">
@@ -6253,7 +6253,7 @@
         <v>-1.86</v>
       </c>
       <c r="G185" t="n">
-        <v>9.05116432820149</v>
+        <v>15.1591701366004</v>
       </c>
     </row>
     <row r="186">
@@ -6276,7 +6276,7 @@
         <v>-6.6</v>
       </c>
       <c r="G186" t="n">
-        <v>2.92975148749568</v>
+        <v>4.19624685630788</v>
       </c>
     </row>
     <row r="187">
@@ -6299,7 +6299,7 @@
         <v>-5.99</v>
       </c>
       <c r="G187" t="n">
-        <v>4.65070060310209</v>
+        <v>4.29871390597615</v>
       </c>
     </row>
     <row r="188">
@@ -6322,7 +6322,7 @@
         <v>-0.48</v>
       </c>
       <c r="G188" t="n">
-        <v>2.81999014682214</v>
+        <v>4.71329199026656</v>
       </c>
     </row>
     <row r="189">
@@ -6414,7 +6414,7 @@
         <v>274.62</v>
       </c>
       <c r="G192" t="n">
-        <v>-230.62</v>
+        <v>-4976.14028062427</v>
       </c>
     </row>
     <row r="193">
@@ -6483,7 +6483,7 @@
         <v>-73.1099999999997</v>
       </c>
       <c r="G195" t="n">
-        <v>-4289.30402798378</v>
+        <v>-205.782142857143</v>
       </c>
     </row>
     <row r="196">
@@ -6598,7 +6598,7 @@
         <v>-2646.36</v>
       </c>
       <c r="G200" t="n">
-        <v>777.140725195117</v>
+        <v>728.616729522345</v>
       </c>
     </row>
     <row r="201">
@@ -6943,7 +6943,7 @@
         <v>-2305.05</v>
       </c>
       <c r="G215" t="n">
-        <v>1003.30579916612</v>
+        <v>909.019204299993</v>
       </c>
     </row>
     <row r="216">
@@ -7035,7 +7035,7 @@
         <v>1.706</v>
       </c>
       <c r="G219" t="n">
-        <v>0.82429014531241</v>
+        <v>1.48473335519028</v>
       </c>
     </row>
     <row r="220">
@@ -7058,7 +7058,7 @@
         <v>4.218</v>
       </c>
       <c r="G220" t="n">
-        <v>1.19750703669354</v>
+        <v>1.80730259967167</v>
       </c>
     </row>
     <row r="221">
@@ -7081,7 +7081,7 @@
         <v>1.578</v>
       </c>
       <c r="G221" t="n">
-        <v>0.681453961726472</v>
+        <v>1.05004537447068</v>
       </c>
     </row>
     <row r="222">
@@ -7104,7 +7104,7 @@
         <v>3.683</v>
       </c>
       <c r="G222" t="n">
-        <v>5.58673345802865</v>
+        <v>4.95769449454787</v>
       </c>
     </row>
     <row r="223">
@@ -7127,7 +7127,7 @@
         <v>2.983</v>
       </c>
       <c r="G223" t="n">
-        <v>7.83348756962292</v>
+        <v>5.0599107657216</v>
       </c>
     </row>
     <row r="224">
@@ -7150,7 +7150,7 @@
         <v>2.44</v>
       </c>
       <c r="G224" t="n">
-        <v>2.65063959823167</v>
+        <v>2.42722772642028</v>
       </c>
     </row>
     <row r="225">
@@ -7173,7 +7173,7 @@
         <v>3.879</v>
       </c>
       <c r="G225" t="n">
-        <v>0.994453725405244</v>
+        <v>6.02384314952086</v>
       </c>
     </row>
     <row r="226">
@@ -7196,7 +7196,7 @@
         <v>0.579999999999998</v>
       </c>
       <c r="G226" t="n">
-        <v>0.249356137630547</v>
+        <v>0.987742431407015</v>
       </c>
     </row>
     <row r="227">
@@ -7219,7 +7219,7 @@
         <v>-1.918</v>
       </c>
       <c r="G227" t="n">
-        <v>-0.519816745809801</v>
+        <v>-0.716224489338153</v>
       </c>
     </row>
     <row r="228">
@@ -7242,7 +7242,7 @@
         <v>0.672000000000001</v>
       </c>
       <c r="G228" t="n">
-        <v>0.6537835233477</v>
+        <v>1.11839214030449</v>
       </c>
     </row>
     <row r="229">
@@ -7265,7 +7265,7 @@
         <v>0.352999999999998</v>
       </c>
       <c r="G229" t="n">
-        <v>0.969100798857603</v>
+        <v>-0.0216294844515644</v>
       </c>
     </row>
     <row r="230">
@@ -7288,7 +7288,7 @@
         <v>5.08900000000001</v>
       </c>
       <c r="G230" t="n">
-        <v>3.26566933983735</v>
+        <v>3.54271097718499</v>
       </c>
     </row>
     <row r="231">
@@ -7311,7 +7311,7 @@
         <v>0.181000000000001</v>
       </c>
       <c r="G231" t="n">
-        <v>-4.30888341671657</v>
+        <v>1.57683280022581</v>
       </c>
     </row>
     <row r="232">
@@ -7334,7 +7334,7 @@
         <v>1.311</v>
       </c>
       <c r="G232" t="n">
-        <v>0.985545683553307</v>
+        <v>1.75135883473944</v>
       </c>
     </row>
     <row r="233">
@@ -7357,7 +7357,7 @@
         <v>2.862</v>
       </c>
       <c r="G233" t="n">
-        <v>2.77429923741266</v>
+        <v>1.43373191636847</v>
       </c>
     </row>
     <row r="234">
@@ -7380,7 +7380,7 @@
         <v>54</v>
       </c>
       <c r="G234" t="n">
-        <v>33.7705105442409</v>
+        <v>40.4285714285714</v>
       </c>
     </row>
     <row r="235">
@@ -7403,7 +7403,7 @@
         <v>83</v>
       </c>
       <c r="G235" t="n">
-        <v>30.5516459075398</v>
+        <v>38.3571428571429</v>
       </c>
     </row>
     <row r="236">
@@ -7426,7 +7426,7 @@
         <v>90</v>
       </c>
       <c r="G236" t="n">
-        <v>36.9003057807971</v>
+        <v>7.21448610215936</v>
       </c>
     </row>
     <row r="237">
@@ -7449,7 +7449,7 @@
         <v>35</v>
       </c>
       <c r="G237" t="n">
-        <v>46.4760733114377</v>
+        <v>41.7857142857143</v>
       </c>
     </row>
     <row r="238">
@@ -7472,7 +7472,7 @@
         <v>5</v>
       </c>
       <c r="G238" t="n">
-        <v>85.0619895397796</v>
+        <v>79.8994457637627</v>
       </c>
     </row>
     <row r="239">
@@ -7518,7 +7518,7 @@
         <v>25</v>
       </c>
       <c r="G240" t="n">
-        <v>-68.5137678121679</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="241">
@@ -7564,7 +7564,7 @@
         <v>49</v>
       </c>
       <c r="G242" t="n">
-        <v>40.1117646073871</v>
+        <v>40.7857142857143</v>
       </c>
     </row>
     <row r="243">
@@ -7633,7 +7633,7 @@
         <v>25</v>
       </c>
       <c r="G245" t="n">
-        <v>50.972887912527</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="246">
@@ -7656,7 +7656,7 @@
         <v>18</v>
       </c>
       <c r="G246" t="n">
-        <v>87.7835041764773</v>
+        <v>52.7338385740492</v>
       </c>
     </row>
     <row r="247">
@@ -7840,7 +7840,7 @@
         <v>23</v>
       </c>
       <c r="G254" t="n">
-        <v>6.94459873105832</v>
+        <v>8.92307692307692</v>
       </c>
     </row>
     <row r="255">
@@ -7886,7 +7886,7 @@
         <v>20</v>
       </c>
       <c r="G256" t="n">
-        <v>9.15384615384616</v>
+        <v>7.50189888343359</v>
       </c>
     </row>
     <row r="257">
@@ -7955,7 +7955,7 @@
         <v>16</v>
       </c>
       <c r="G259" t="n">
-        <v>9.41177712977729</v>
+        <v>9.46153846153846</v>
       </c>
     </row>
     <row r="260">
@@ -8047,7 +8047,7 @@
         <v>9.43</v>
       </c>
       <c r="G263" t="n">
-        <v>-7.30645795590716</v>
+        <v>-10.6448443175743</v>
       </c>
     </row>
     <row r="264">
@@ -8070,7 +8070,7 @@
         <v>20.73</v>
       </c>
       <c r="G264" t="n">
-        <v>4.82148826149735</v>
+        <v>3.92052542828579</v>
       </c>
     </row>
     <row r="265">
@@ -8093,7 +8093,7 @@
         <v>13.69</v>
       </c>
       <c r="G265" t="n">
-        <v>3.61810199164956</v>
+        <v>8.18062345814712</v>
       </c>
     </row>
     <row r="266">
@@ -8116,7 +8116,7 @@
         <v>10.45</v>
       </c>
       <c r="G266" t="n">
-        <v>1.73222948458399</v>
+        <v>2.78938737974451</v>
       </c>
     </row>
     <row r="267">
@@ -8139,7 +8139,7 @@
         <v>14.93</v>
       </c>
       <c r="G267" t="n">
-        <v>5.75750439431132</v>
+        <v>7.05753260968619</v>
       </c>
     </row>
     <row r="268">
@@ -8162,7 +8162,7 @@
         <v>13.79</v>
       </c>
       <c r="G268" t="n">
-        <v>2.264681353266</v>
+        <v>2.87125907402235</v>
       </c>
     </row>
     <row r="269">
@@ -8185,7 +8185,7 @@
         <v>13.72</v>
       </c>
       <c r="G269" t="n">
-        <v>9.95347767232906</v>
+        <v>7.93624055196986</v>
       </c>
     </row>
     <row r="270">
@@ -8208,7 +8208,7 @@
         <v>0.79</v>
       </c>
       <c r="G270" t="n">
-        <v>16.1249204952411</v>
+        <v>14.6969673146841</v>
       </c>
     </row>
     <row r="271">
@@ -8231,7 +8231,7 @@
         <v>0.85</v>
       </c>
       <c r="G271" t="n">
-        <v>5.03349777229473</v>
+        <v>7.43772521365648</v>
       </c>
     </row>
     <row r="272">
@@ -8254,7 +8254,7 @@
         <v>-4.09</v>
       </c>
       <c r="G272" t="n">
-        <v>7.33857771903703</v>
+        <v>7.05090668681676</v>
       </c>
     </row>
     <row r="273">
@@ -8277,7 +8277,7 @@
         <v>-0.74</v>
       </c>
       <c r="G273" t="n">
-        <v>3.13098414394587</v>
+        <v>2.93221956096258</v>
       </c>
     </row>
     <row r="274">
@@ -8300,7 +8300,7 @@
         <v>-1.86</v>
       </c>
       <c r="G274" t="n">
-        <v>7.54498274705035</v>
+        <v>6.99122343860655</v>
       </c>
     </row>
     <row r="275">
@@ -8323,7 +8323,7 @@
         <v>-6.6</v>
       </c>
       <c r="G275" t="n">
-        <v>1.30146566566075</v>
+        <v>2.41981005376708</v>
       </c>
     </row>
     <row r="276">
@@ -8346,7 +8346,7 @@
         <v>-5.99</v>
       </c>
       <c r="G276" t="n">
-        <v>10.5359508536538</v>
+        <v>9.40337078085868</v>
       </c>
     </row>
     <row r="277">
@@ -8369,7 +8369,7 @@
         <v>-0.48</v>
       </c>
       <c r="G277" t="n">
-        <v>1.58957205928497</v>
+        <v>2.07494219622767</v>
       </c>
     </row>
     <row r="278">
@@ -8392,7 +8392,7 @@
         <v>874.31</v>
       </c>
       <c r="G278" t="n">
-        <v>-1434.83246758494</v>
+        <v>-1955.08022600621</v>
       </c>
     </row>
     <row r="279">
@@ -8415,7 +8415,7 @@
         <v>1757.71</v>
       </c>
       <c r="G279" t="n">
-        <v>362.632537428349</v>
+        <v>230.996634911877</v>
       </c>
     </row>
     <row r="280">
@@ -8438,7 +8438,7 @@
         <v>1924.77</v>
       </c>
       <c r="G280" t="n">
-        <v>-1145.06260160065</v>
+        <v>-157.71487340053</v>
       </c>
     </row>
     <row r="281">
@@ -8461,7 +8461,7 @@
         <v>274.62</v>
       </c>
       <c r="G281" t="n">
-        <v>-629.63013163342</v>
+        <v>-702.420369387117</v>
       </c>
     </row>
     <row r="282">
@@ -8484,7 +8484,7 @@
         <v>545.54</v>
       </c>
       <c r="G282" t="n">
-        <v>-249.061999887392</v>
+        <v>2.24604282448442</v>
       </c>
     </row>
     <row r="283">
@@ -8507,7 +8507,7 @@
         <v>1276.8</v>
       </c>
       <c r="G283" t="n">
-        <v>-1356.64235005597</v>
+        <v>-1227.96381443763</v>
       </c>
     </row>
     <row r="284">
@@ -8530,7 +8530,7 @@
         <v>535.780000000001</v>
       </c>
       <c r="G284" t="n">
-        <v>1096.91912639863</v>
+        <v>945.275879024311</v>
       </c>
     </row>
     <row r="285">
@@ -8553,7 +8553,7 @@
         <v>171.549999999999</v>
       </c>
       <c r="G285" t="n">
-        <v>1257.85686056013</v>
+        <v>1291.90527978315</v>
       </c>
     </row>
     <row r="286">
@@ -8576,7 +8576,7 @@
         <v>621.64</v>
       </c>
       <c r="G286" t="n">
-        <v>-204.422216916147</v>
+        <v>103.791324762464</v>
       </c>
     </row>
     <row r="287">
@@ -8599,7 +8599,7 @@
         <v>-1588.06</v>
       </c>
       <c r="G287" t="n">
-        <v>486.96959194571</v>
+        <v>515.113025704633</v>
       </c>
     </row>
     <row r="288">
@@ -8622,7 +8622,7 @@
         <v>-845.39</v>
       </c>
       <c r="G288" t="n">
-        <v>-82.1244017684587</v>
+        <v>-167.56818110796</v>
       </c>
     </row>
     <row r="289">
@@ -8645,7 +8645,7 @@
         <v>-2646.36</v>
       </c>
       <c r="G289" t="n">
-        <v>178.364224481377</v>
+        <v>74.7783247599603</v>
       </c>
     </row>
     <row r="290">
@@ -8668,7 +8668,7 @@
         <v>-1385.12</v>
       </c>
       <c r="G290" t="n">
-        <v>-759.262726433839</v>
+        <v>-880.324610592611</v>
       </c>
     </row>
     <row r="291">
@@ -8691,7 +8691,7 @@
         <v>-2594.04</v>
       </c>
       <c r="G291" t="n">
-        <v>741.381059309979</v>
+        <v>389.913154940841</v>
       </c>
     </row>
     <row r="292">
@@ -8714,7 +8714,7 @@
         <v>-1268.92</v>
       </c>
       <c r="G292" t="n">
-        <v>-583.495248563769</v>
+        <v>-657.715406834633</v>
       </c>
     </row>
     <row r="293">
@@ -8737,7 +8737,7 @@
         <v>517.34</v>
       </c>
       <c r="G293" t="n">
-        <v>-931.577211335378</v>
+        <v>-1464.48025759576</v>
       </c>
     </row>
     <row r="294">
@@ -8760,7 +8760,7 @@
         <v>1517.85</v>
       </c>
       <c r="G294" t="n">
-        <v>520.223223838638</v>
+        <v>487.549433701524</v>
       </c>
     </row>
     <row r="295">
@@ -8783,7 +8783,7 @@
         <v>2790.83</v>
       </c>
       <c r="G295" t="n">
-        <v>-452.365104825049</v>
+        <v>126.4744327656</v>
       </c>
     </row>
     <row r="296">
@@ -8806,7 +8806,7 @@
         <v>739.459999999999</v>
       </c>
       <c r="G296" t="n">
-        <v>-622.208959343092</v>
+        <v>-631.914833825956</v>
       </c>
     </row>
     <row r="297">
@@ -8829,7 +8829,7 @@
         <v>1179</v>
       </c>
       <c r="G297" t="n">
-        <v>96.5144822609254</v>
+        <v>301.614525320721</v>
       </c>
     </row>
     <row r="298">
@@ -8852,7 +8852,7 @@
         <v>682.55</v>
       </c>
       <c r="G298" t="n">
-        <v>-748.857924744324</v>
+        <v>-549.59595230943</v>
       </c>
     </row>
     <row r="299">
@@ -8875,7 +8875,7 @@
         <v>882.37</v>
       </c>
       <c r="G299" t="n">
-        <v>1023.49552407212</v>
+        <v>1042.07042808988</v>
       </c>
     </row>
     <row r="300">
@@ -8898,7 +8898,7 @@
         <v>-171.76</v>
       </c>
       <c r="G300" t="n">
-        <v>1559.15955836404</v>
+        <v>1689.11748196996</v>
       </c>
     </row>
     <row r="301">
@@ -8921,7 +8921,7 @@
         <v>854.04</v>
       </c>
       <c r="G301" t="n">
-        <v>-13.2224096404099</v>
+        <v>270.805436884527</v>
       </c>
     </row>
     <row r="302">
@@ -8944,7 +8944,7 @@
         <v>-1503.6</v>
       </c>
       <c r="G302" t="n">
-        <v>748.508148022878</v>
+        <v>752.667823190055</v>
       </c>
     </row>
     <row r="303">
@@ -8967,7 +8967,7 @@
         <v>-88.7199999999993</v>
       </c>
       <c r="G303" t="n">
-        <v>8.91038175380643</v>
+        <v>-127.889486280421</v>
       </c>
     </row>
     <row r="304">
@@ -8990,7 +8990,7 @@
         <v>-2305.05</v>
       </c>
       <c r="G304" t="n">
-        <v>286.474741112046</v>
+        <v>223.263797155856</v>
       </c>
     </row>
     <row r="305">
@@ -9013,7 +9013,7 @@
         <v>-1179.58</v>
       </c>
       <c r="G305" t="n">
-        <v>-742.238785639724</v>
+        <v>-827.736166473996</v>
       </c>
     </row>
     <row r="306">
@@ -9036,7 +9036,7 @@
         <v>-1491.94</v>
       </c>
       <c r="G306" t="n">
-        <v>1166.70499516399</v>
+        <v>616.0028260033</v>
       </c>
     </row>
     <row r="307">
@@ -9059,7 +9059,7 @@
         <v>-1081</v>
       </c>
       <c r="G307" t="n">
-        <v>-345.148460257647</v>
+        <v>-370.614253247223</v>
       </c>
     </row>
     <row r="308">
@@ -9082,7 +9082,7 @@
         <v>1.706</v>
       </c>
       <c r="G308" t="n">
-        <v>0.258925025826104</v>
+        <v>0.801452465375178</v>
       </c>
     </row>
     <row r="309">
@@ -9105,7 +9105,7 @@
         <v>4.218</v>
       </c>
       <c r="G309" t="n">
-        <v>0.631173392985819</v>
+        <v>0.56603225111432</v>
       </c>
     </row>
     <row r="310">
@@ -9128,7 +9128,7 @@
         <v>1.578</v>
       </c>
       <c r="G310" t="n">
-        <v>2.29375532420241</v>
+        <v>2.51734362624757</v>
       </c>
     </row>
     <row r="311">
@@ -9151,7 +9151,7 @@
         <v>3.683</v>
       </c>
       <c r="G311" t="n">
-        <v>2.07417284390818</v>
+        <v>2.76889688081292</v>
       </c>
     </row>
     <row r="312">
@@ -9174,7 +9174,7 @@
         <v>2.983</v>
       </c>
       <c r="G312" t="n">
-        <v>2.41732430648026</v>
+        <v>2.34856119970111</v>
       </c>
     </row>
     <row r="313">
@@ -9197,7 +9197,7 @@
         <v>2.44</v>
       </c>
       <c r="G313" t="n">
-        <v>4.31017205918876</v>
+        <v>3.64649306909352</v>
       </c>
     </row>
     <row r="314">
@@ -9220,7 +9220,7 @@
         <v>3.614</v>
       </c>
       <c r="G314" t="n">
-        <v>1.38364166353821</v>
+        <v>0.951503924548786</v>
       </c>
     </row>
     <row r="315">
@@ -9243,7 +9243,7 @@
         <v>0.579999999999998</v>
       </c>
       <c r="G315" t="n">
-        <v>2.68228049726895</v>
+        <v>1.8594822707144</v>
       </c>
     </row>
     <row r="316">
@@ -9266,7 +9266,7 @@
         <v>-1.918</v>
       </c>
       <c r="G316" t="n">
-        <v>1.78887071777641</v>
+        <v>2.0698046038911</v>
       </c>
     </row>
     <row r="317">
@@ -9289,7 +9289,7 @@
         <v>0.672000000000001</v>
       </c>
       <c r="G317" t="n">
-        <v>0.811436534124472</v>
+        <v>0.761926078957812</v>
       </c>
     </row>
     <row r="318">
@@ -9312,7 +9312,7 @@
         <v>0.352999999999998</v>
       </c>
       <c r="G318" t="n">
-        <v>0.476807058062741</v>
+        <v>0.80486203620573</v>
       </c>
     </row>
     <row r="319">
@@ -9335,7 +9335,7 @@
         <v>5.08900000000001</v>
       </c>
       <c r="G319" t="n">
-        <v>2.38363857153648</v>
+        <v>2.27515468959244</v>
       </c>
     </row>
     <row r="320">
@@ -9358,7 +9358,7 @@
         <v>0.181000000000001</v>
       </c>
       <c r="G320" t="n">
-        <v>2.66084602254892</v>
+        <v>2.79079802742034</v>
       </c>
     </row>
     <row r="321">
@@ -9381,7 +9381,7 @@
         <v>1.311</v>
       </c>
       <c r="G321" t="n">
-        <v>2.12987792246682</v>
+        <v>2.34863191891748</v>
       </c>
     </row>
     <row r="322">
@@ -9404,7 +9404,7 @@
         <v>2.862</v>
       </c>
       <c r="G322" t="n">
-        <v>1.5917509464141</v>
+        <v>1.81486148813662</v>
       </c>
     </row>
     <row r="323">
@@ -9427,7 +9427,7 @@
         <v>54</v>
       </c>
       <c r="G323" t="n">
-        <v>45.1430663105095</v>
+        <v>46.0855745068511</v>
       </c>
     </row>
     <row r="324">
@@ -9450,7 +9450,7 @@
         <v>83</v>
       </c>
       <c r="G324" t="n">
-        <v>61.0525731208162</v>
+        <v>57.7529938870765</v>
       </c>
     </row>
     <row r="325">
@@ -9473,7 +9473,7 @@
         <v>90</v>
       </c>
       <c r="G325" t="n">
-        <v>21.011166274585</v>
+        <v>33.355772861997</v>
       </c>
     </row>
     <row r="326">
@@ -9496,7 +9496,7 @@
         <v>35</v>
       </c>
       <c r="G326" t="n">
-        <v>24.7611314122024</v>
+        <v>21.2629266390353</v>
       </c>
     </row>
     <row r="327">
@@ -9519,7 +9519,7 @@
         <v>5</v>
       </c>
       <c r="G327" t="n">
-        <v>46.2168459628802</v>
+        <v>47.7909381503857</v>
       </c>
     </row>
     <row r="328">
@@ -9542,7 +9542,7 @@
         <v>3</v>
       </c>
       <c r="G328" t="n">
-        <v>25.0262776833676</v>
+        <v>26.2649090588523</v>
       </c>
     </row>
     <row r="329">
@@ -9565,7 +9565,7 @@
         <v>65</v>
       </c>
       <c r="G329" t="n">
-        <v>61.7447815196297</v>
+        <v>61.7229252613714</v>
       </c>
     </row>
     <row r="330">
@@ -9588,7 +9588,7 @@
         <v>72</v>
       </c>
       <c r="G330" t="n">
-        <v>55.0915667829143</v>
+        <v>58.8112025467463</v>
       </c>
     </row>
     <row r="331">
@@ -9611,7 +9611,7 @@
         <v>49</v>
       </c>
       <c r="G331" t="n">
-        <v>51.5681539442287</v>
+        <v>51.4525998155861</v>
       </c>
     </row>
     <row r="332">
@@ -9634,7 +9634,7 @@
         <v>5</v>
       </c>
       <c r="G332" t="n">
-        <v>72.2633277213891</v>
+        <v>71.2294513654726</v>
       </c>
     </row>
     <row r="333">
@@ -9657,7 +9657,7 @@
         <v>62</v>
       </c>
       <c r="G333" t="n">
-        <v>52.9121460199706</v>
+        <v>54.197327327089</v>
       </c>
     </row>
     <row r="334">
@@ -9680,7 +9680,7 @@
         <v>25</v>
       </c>
       <c r="G334" t="n">
-        <v>10.3895262768893</v>
+        <v>10.0216994777284</v>
       </c>
     </row>
     <row r="335">
@@ -9703,7 +9703,7 @@
         <v>18</v>
       </c>
       <c r="G335" t="n">
-        <v>43.9473983903037</v>
+        <v>43.1280602083368</v>
       </c>
     </row>
     <row r="336">
@@ -9726,7 +9726,7 @@
         <v>5</v>
       </c>
       <c r="G336" t="n">
-        <v>51.1883543110375</v>
+        <v>48.6905167005712</v>
       </c>
     </row>
     <row r="337">
@@ -9749,7 +9749,7 @@
         <v>89</v>
       </c>
       <c r="G337" t="n">
-        <v>24.7034464507733</v>
+        <v>26.3453593624658</v>
       </c>
     </row>
     <row r="338">
@@ -9772,7 +9772,7 @@
         <v>5</v>
       </c>
       <c r="G338" t="n">
-        <v>-0.428282039140081</v>
+        <v>-1.81969291421405</v>
       </c>
     </row>
     <row r="339">
@@ -9795,7 +9795,7 @@
         <v>14</v>
       </c>
       <c r="G339" t="n">
-        <v>8.40875438192256</v>
+        <v>9.06335331294624</v>
       </c>
     </row>
     <row r="340">
@@ -9818,7 +9818,7 @@
         <v>4</v>
       </c>
       <c r="G340" t="n">
-        <v>13.1773695647422</v>
+        <v>12.3847322556698</v>
       </c>
     </row>
     <row r="341">
@@ -9841,7 +9841,7 @@
         <v>11</v>
       </c>
       <c r="G341" t="n">
-        <v>12.3642776404871</v>
+        <v>12.917151983823</v>
       </c>
     </row>
     <row r="342">
@@ -9864,7 +9864,7 @@
         <v>10</v>
       </c>
       <c r="G342" t="n">
-        <v>10.8278139523967</v>
+        <v>11.1154929928391</v>
       </c>
     </row>
     <row r="343">
@@ -9887,7 +9887,7 @@
         <v>8</v>
       </c>
       <c r="G343" t="n">
-        <v>12.3271563832538</v>
+        <v>12.1937638009104</v>
       </c>
     </row>
     <row r="344">
@@ -9910,7 +9910,7 @@
         <v>6</v>
       </c>
       <c r="G344" t="n">
-        <v>11.5457703916747</v>
+        <v>11.5181563848875</v>
       </c>
     </row>
     <row r="345">
@@ -9933,7 +9933,7 @@
         <v>20</v>
       </c>
       <c r="G345" t="n">
-        <v>8.05346594154424</v>
+        <v>8.54763621214285</v>
       </c>
     </row>
     <row r="346">
@@ -9956,7 +9956,7 @@
         <v>7</v>
       </c>
       <c r="G346" t="n">
-        <v>10.168917482822</v>
+        <v>9.37853363584052</v>
       </c>
     </row>
     <row r="347">
@@ -9979,7 +9979,7 @@
         <v>6</v>
       </c>
       <c r="G347" t="n">
-        <v>8.24342620802681</v>
+        <v>7.9950396760771</v>
       </c>
     </row>
     <row r="348">
@@ -10002,7 +10002,7 @@
         <v>16</v>
       </c>
       <c r="G348" t="n">
-        <v>7.95824150999623</v>
+        <v>7.6680352131873</v>
       </c>
     </row>
     <row r="349">
@@ -10025,7 +10025,7 @@
         <v>1</v>
       </c>
       <c r="G349" t="n">
-        <v>5.4871304643102</v>
+        <v>5.24922842582923</v>
       </c>
     </row>
     <row r="350">
@@ -10048,7 +10048,7 @@
         <v>15</v>
       </c>
       <c r="G350" t="n">
-        <v>7.87297295908987</v>
+        <v>6.96815975413788</v>
       </c>
     </row>
     <row r="351">
@@ -10071,7 +10071,7 @@
         <v>1</v>
       </c>
       <c r="G351" t="n">
-        <v>8.03935696481911</v>
+        <v>7.87305195529037</v>
       </c>
     </row>
     <row r="352">
@@ -10094,7 +10094,7 @@
         <v>9.43</v>
       </c>
       <c r="G352" t="n">
-        <v>0.463419222357327</v>
+        <v>-2.53824521290242</v>
       </c>
     </row>
     <row r="353">
@@ -10117,7 +10117,7 @@
         <v>20.73</v>
       </c>
       <c r="G353" t="n">
-        <v>-0.592850891323601</v>
+        <v>-0.202569013670269</v>
       </c>
     </row>
     <row r="354">
@@ -10140,7 +10140,7 @@
         <v>13.69</v>
       </c>
       <c r="G354" t="n">
-        <v>-11.2312193457404</v>
+        <v>1.48704484280394</v>
       </c>
     </row>
     <row r="355">
@@ -10163,7 +10163,7 @@
         <v>10.45</v>
       </c>
       <c r="G355" t="n">
-        <v>5.9237596016223</v>
+        <v>8.46009062001433</v>
       </c>
     </row>
     <row r="356">
@@ -10186,7 +10186,7 @@
         <v>14.93</v>
       </c>
       <c r="G356" t="n">
-        <v>2.6830533563006</v>
+        <v>3.04426769236808</v>
       </c>
     </row>
     <row r="357">
@@ -10209,7 +10209,7 @@
         <v>13.79</v>
       </c>
       <c r="G357" t="n">
-        <v>0.333152394263345</v>
+        <v>1.28326319286417</v>
       </c>
     </row>
     <row r="358">
@@ -10232,7 +10232,7 @@
         <v>0.79</v>
       </c>
       <c r="G358" t="n">
-        <v>11.0391510294654</v>
+        <v>12.9128679493924</v>
       </c>
     </row>
     <row r="359">
@@ -10255,7 +10255,7 @@
         <v>0.85</v>
       </c>
       <c r="G359" t="n">
-        <v>4.86324564357585</v>
+        <v>6.30989940583107</v>
       </c>
     </row>
     <row r="360">
@@ -10278,7 +10278,7 @@
         <v>-4.09</v>
       </c>
       <c r="G360" t="n">
-        <v>10.0450644799623</v>
+        <v>8.72507583855613</v>
       </c>
     </row>
     <row r="361">
@@ -10301,7 +10301,7 @@
         <v>-0.74</v>
       </c>
       <c r="G361" t="n">
-        <v>4.77765907094509</v>
+        <v>4.44683949347272</v>
       </c>
     </row>
     <row r="362">
@@ -10324,7 +10324,7 @@
         <v>-1.86</v>
       </c>
       <c r="G362" t="n">
-        <v>7.31289315151617</v>
+        <v>7.25563435047662</v>
       </c>
     </row>
     <row r="363">
@@ -10347,7 +10347,7 @@
         <v>-6.6</v>
       </c>
       <c r="G363" t="n">
-        <v>5.74291045249566</v>
+        <v>4.0005797255714</v>
       </c>
     </row>
     <row r="364">
@@ -10370,7 +10370,7 @@
         <v>-5.99</v>
       </c>
       <c r="G364" t="n">
-        <v>10.3028996389021</v>
+        <v>9.02186575093266</v>
       </c>
     </row>
     <row r="365">
@@ -10393,7 +10393,7 @@
         <v>-0.48</v>
       </c>
       <c r="G365" t="n">
-        <v>7.68394875827547</v>
+        <v>6.34345020704452</v>
       </c>
     </row>
     <row r="366">
@@ -10416,7 +10416,7 @@
         <v>874.31</v>
       </c>
       <c r="G366" t="n">
-        <v>-1215.79540870551</v>
+        <v>-1559.87980137917</v>
       </c>
     </row>
     <row r="367">
@@ -10439,7 +10439,7 @@
         <v>1757.71</v>
       </c>
       <c r="G367" t="n">
-        <v>-364.195795748132</v>
+        <v>-325.384561038346</v>
       </c>
     </row>
     <row r="368">
@@ -10462,7 +10462,7 @@
         <v>1924.77</v>
       </c>
       <c r="G368" t="n">
-        <v>-969.860103760024</v>
+        <v>-327.713770214601</v>
       </c>
     </row>
     <row r="369">
@@ -10485,7 +10485,7 @@
         <v>274.62</v>
       </c>
       <c r="G369" t="n">
-        <v>132.633966169134</v>
+        <v>431.472495992092</v>
       </c>
     </row>
     <row r="370">
@@ -10508,7 +10508,7 @@
         <v>545.54</v>
       </c>
       <c r="G370" t="n">
-        <v>218.693115730672</v>
+        <v>206.006536854927</v>
       </c>
     </row>
     <row r="371">
@@ -10531,7 +10531,7 @@
         <v>1276.8</v>
       </c>
       <c r="G371" t="n">
-        <v>-941.517993007494</v>
+        <v>-907.507807933359</v>
       </c>
     </row>
     <row r="372">
@@ -10554,7 +10554,7 @@
         <v>171.549999999999</v>
       </c>
       <c r="G372" t="n">
-        <v>922.62281548384</v>
+        <v>1173.97673534793</v>
       </c>
     </row>
     <row r="373">
@@ -10577,7 +10577,7 @@
         <v>621.64</v>
       </c>
       <c r="G373" t="n">
-        <v>-265.192158869579</v>
+        <v>-245.231554790478</v>
       </c>
     </row>
     <row r="374">
@@ -10600,7 +10600,7 @@
         <v>-1588.06</v>
       </c>
       <c r="G374" t="n">
-        <v>836.166876874522</v>
+        <v>536.2699334114</v>
       </c>
     </row>
     <row r="375">
@@ -10623,7 +10623,7 @@
         <v>-845.39</v>
       </c>
       <c r="G375" t="n">
-        <v>-243.234892128579</v>
+        <v>-270.41683691112</v>
       </c>
     </row>
     <row r="376">
@@ -10646,7 +10646,7 @@
         <v>-2646.36</v>
       </c>
       <c r="G376" t="n">
-        <v>-120.13056220682</v>
+        <v>-23.0125103358143</v>
       </c>
     </row>
     <row r="377">
@@ -10669,7 +10669,7 @@
         <v>-1385.12</v>
       </c>
       <c r="G377" t="n">
-        <v>-71.7735052103275</v>
+        <v>-233.199194901478</v>
       </c>
     </row>
     <row r="378">
@@ -10692,7 +10692,7 @@
         <v>-2594.04</v>
       </c>
       <c r="G378" t="n">
-        <v>948.22754044915</v>
+        <v>572.226311502931</v>
       </c>
     </row>
     <row r="379">
@@ -10715,7 +10715,7 @@
         <v>-1268.92</v>
       </c>
       <c r="G379" t="n">
-        <v>7.6431808906369</v>
+        <v>39.7836033264657</v>
       </c>
     </row>
     <row r="380">
@@ -10738,7 +10738,7 @@
         <v>517.34</v>
       </c>
       <c r="G380" t="n">
-        <v>-673.168980122582</v>
+        <v>-937.006134606962</v>
       </c>
     </row>
     <row r="381">
@@ -10761,7 +10761,7 @@
         <v>1517.85</v>
       </c>
       <c r="G381" t="n">
-        <v>90.1684426712062</v>
+        <v>122.061117707073</v>
       </c>
     </row>
     <row r="382">
@@ -10784,7 +10784,7 @@
         <v>2790.83</v>
       </c>
       <c r="G382" t="n">
-        <v>-504.897523833645</v>
+        <v>-57.4721864532361</v>
       </c>
     </row>
     <row r="383">
@@ -10807,7 +10807,7 @@
         <v>739.459999999999</v>
       </c>
       <c r="G383" t="n">
-        <v>40.6032778990432</v>
+        <v>184.369974552123</v>
       </c>
     </row>
     <row r="384">
@@ -10830,7 +10830,7 @@
         <v>1179</v>
       </c>
       <c r="G384" t="n">
-        <v>231.041560706482</v>
+        <v>323.956125476191</v>
       </c>
     </row>
     <row r="385">
@@ -10853,7 +10853,7 @@
         <v>682.55</v>
       </c>
       <c r="G385" t="n">
-        <v>-560.51586986742</v>
+        <v>-465.318108276405</v>
       </c>
     </row>
     <row r="386">
@@ -10876,7 +10876,7 @@
         <v>-171.76</v>
       </c>
       <c r="G386" t="n">
-        <v>1372.27842313172</v>
+        <v>1503.29799330004</v>
       </c>
     </row>
     <row r="387">
@@ -10899,7 +10899,7 @@
         <v>854.04</v>
       </c>
       <c r="G387" t="n">
-        <v>34.980677182863</v>
+        <v>53.3232732492818</v>
       </c>
     </row>
     <row r="388">
@@ -10922,7 +10922,7 @@
         <v>-1503.6</v>
       </c>
       <c r="G388" t="n">
-        <v>986.398671066671</v>
+        <v>723.503498704684</v>
       </c>
     </row>
     <row r="389">
@@ -10945,7 +10945,7 @@
         <v>-88.7199999999993</v>
       </c>
       <c r="G389" t="n">
-        <v>-12.9270538509499</v>
+        <v>-34.0380910425838</v>
       </c>
     </row>
     <row r="390">
@@ -10968,7 +10968,7 @@
         <v>-2305.05</v>
       </c>
       <c r="G390" t="n">
-        <v>-1099.8815178929</v>
+        <v>-899.178565288362</v>
       </c>
     </row>
     <row r="391">
@@ -10991,7 +10991,7 @@
         <v>-1179.58</v>
       </c>
       <c r="G391" t="n">
-        <v>128.396572886529</v>
+        <v>57.3778978213327</v>
       </c>
     </row>
     <row r="392">
@@ -11014,7 +11014,7 @@
         <v>-1491.94</v>
       </c>
       <c r="G392" t="n">
-        <v>1164.18602145858</v>
+        <v>668.517855270208</v>
       </c>
     </row>
     <row r="393">
@@ -11037,7 +11037,7 @@
         <v>-1081</v>
       </c>
       <c r="G393" t="n">
-        <v>161.279384258362</v>
+        <v>232.037850605788</v>
       </c>
     </row>
     <row r="394">
@@ -11060,7 +11060,7 @@
         <v>1.706</v>
       </c>
       <c r="G394" t="n">
-        <v>3.48541086315014</v>
+        <v>3.47044452192769</v>
       </c>
     </row>
     <row r="395">
@@ -11083,7 +11083,7 @@
         <v>4.218</v>
       </c>
       <c r="G395" t="n">
-        <v>0.572037850230735</v>
+        <v>0.593975731277537</v>
       </c>
     </row>
     <row r="396">
@@ -11106,7 +11106,7 @@
         <v>1.578</v>
       </c>
       <c r="G396" t="n">
-        <v>0.763825069781089</v>
+        <v>1.11942176637849</v>
       </c>
     </row>
     <row r="397">
@@ -11129,7 +11129,7 @@
         <v>3.683</v>
       </c>
       <c r="G397" t="n">
-        <v>1.88407537759575</v>
+        <v>1.87826371323951</v>
       </c>
     </row>
     <row r="398">
@@ -11152,7 +11152,7 @@
         <v>2.983</v>
       </c>
       <c r="G398" t="n">
-        <v>0.583832416083258</v>
+        <v>0.697339226266793</v>
       </c>
     </row>
     <row r="399">
@@ -11175,7 +11175,7 @@
         <v>2.44</v>
       </c>
       <c r="G399" t="n">
-        <v>2.75516889369105</v>
+        <v>2.88565511958409</v>
       </c>
     </row>
     <row r="400">
@@ -11198,7 +11198,7 @@
         <v>0.579999999999998</v>
       </c>
       <c r="G400" t="n">
-        <v>0.712272449938738</v>
+        <v>0.6303731766938</v>
       </c>
     </row>
     <row r="401">
@@ -11221,7 +11221,7 @@
         <v>-1.918</v>
       </c>
       <c r="G401" t="n">
-        <v>1.74360123304795</v>
+        <v>1.91239655844685</v>
       </c>
     </row>
     <row r="402">
@@ -11244,7 +11244,7 @@
         <v>0.672000000000001</v>
       </c>
       <c r="G402" t="n">
-        <v>1.22362510619123</v>
+        <v>1.10326214690224</v>
       </c>
     </row>
     <row r="403">
@@ -11267,7 +11267,7 @@
         <v>0.352999999999998</v>
       </c>
       <c r="G403" t="n">
-        <v>1.93508143110673</v>
+        <v>1.96947803681702</v>
       </c>
     </row>
     <row r="404">
@@ -11290,7 +11290,7 @@
         <v>5.08900000000001</v>
       </c>
       <c r="G404" t="n">
-        <v>2.01506937494894</v>
+        <v>1.53179053857672</v>
       </c>
     </row>
     <row r="405">
@@ -11313,7 +11313,7 @@
         <v>0.181000000000001</v>
       </c>
       <c r="G405" t="n">
-        <v>1.86483288799761</v>
+        <v>1.91103652234291</v>
       </c>
     </row>
     <row r="406">
@@ -11336,7 +11336,7 @@
         <v>1.311</v>
       </c>
       <c r="G406" t="n">
-        <v>1.42281415422913</v>
+        <v>1.56254375222174</v>
       </c>
     </row>
     <row r="407">
@@ -11359,7 +11359,7 @@
         <v>2.862</v>
       </c>
       <c r="G407" t="n">
-        <v>2.07968596935336</v>
+        <v>1.95705523988533</v>
       </c>
     </row>
     <row r="408">
@@ -11382,7 +11382,7 @@
         <v>54</v>
       </c>
       <c r="G408" t="n">
-        <v>47.4890990889449</v>
+        <v>40.4209186552374</v>
       </c>
     </row>
     <row r="409">
@@ -11405,7 +11405,7 @@
         <v>83</v>
       </c>
       <c r="G409" t="n">
-        <v>36.1701243779434</v>
+        <v>36.6770398279956</v>
       </c>
     </row>
     <row r="410">
@@ -11428,7 +11428,7 @@
         <v>90</v>
       </c>
       <c r="G410" t="n">
-        <v>40.4878449192584</v>
+        <v>43.3528397158274</v>
       </c>
     </row>
     <row r="411">
@@ -11451,7 +11451,7 @@
         <v>35</v>
       </c>
       <c r="G411" t="n">
-        <v>69.556741925302</v>
+        <v>69.515300251825</v>
       </c>
     </row>
     <row r="412">
@@ -11474,7 +11474,7 @@
         <v>5</v>
       </c>
       <c r="G412" t="n">
-        <v>48.8732912658077</v>
+        <v>50.8185190684541</v>
       </c>
     </row>
     <row r="413">
@@ -11497,7 +11497,7 @@
         <v>3</v>
       </c>
       <c r="G413" t="n">
-        <v>38.8506454535449</v>
+        <v>39.4870695692717</v>
       </c>
     </row>
     <row r="414">
@@ -11520,7 +11520,7 @@
         <v>72</v>
       </c>
       <c r="G414" t="n">
-        <v>48.4910632905092</v>
+        <v>52.9229837419558</v>
       </c>
     </row>
     <row r="415">
@@ -11543,7 +11543,7 @@
         <v>49</v>
       </c>
       <c r="G415" t="n">
-        <v>36.6958596094381</v>
+        <v>40.9613561030898</v>
       </c>
     </row>
     <row r="416">
@@ -11566,7 +11566,7 @@
         <v>5</v>
       </c>
       <c r="G416" t="n">
-        <v>74.5570325977186</v>
+        <v>72.1831273395868</v>
       </c>
     </row>
     <row r="417">
@@ -11589,7 +11589,7 @@
         <v>62</v>
       </c>
       <c r="G417" t="n">
-        <v>34.1213006388208</v>
+        <v>35.535055652417</v>
       </c>
     </row>
     <row r="418">
@@ -11612,7 +11612,7 @@
         <v>25</v>
       </c>
       <c r="G418" t="n">
-        <v>-16.5167223687251</v>
+        <v>-37.8163724563694</v>
       </c>
     </row>
     <row r="419">
@@ -11635,7 +11635,7 @@
         <v>18</v>
       </c>
       <c r="G419" t="n">
-        <v>39.2794458454653</v>
+        <v>38.2125795368565</v>
       </c>
     </row>
     <row r="420">
@@ -11658,7 +11658,7 @@
         <v>5</v>
       </c>
       <c r="G420" t="n">
-        <v>85.1573121153999</v>
+        <v>67.7156314974068</v>
       </c>
     </row>
     <row r="421">
@@ -11681,7 +11681,7 @@
         <v>89</v>
       </c>
       <c r="G421" t="n">
-        <v>42.8215735082716</v>
+        <v>44.7430173529231</v>
       </c>
     </row>
     <row r="422">
@@ -11704,7 +11704,7 @@
         <v>5</v>
       </c>
       <c r="G422" t="n">
-        <v>0.244333475951734</v>
+        <v>0.738726798737297</v>
       </c>
     </row>
     <row r="423">
@@ -11727,7 +11727,7 @@
         <v>14</v>
       </c>
       <c r="G423" t="n">
-        <v>7.7916168786306</v>
+        <v>9.06342163120697</v>
       </c>
     </row>
     <row r="424">
@@ -11750,7 +11750,7 @@
         <v>4</v>
       </c>
       <c r="G424" t="n">
-        <v>8.28602154887372</v>
+        <v>8.45558036568282</v>
       </c>
     </row>
     <row r="425">
@@ -11773,7 +11773,7 @@
         <v>11</v>
       </c>
       <c r="G425" t="n">
-        <v>11.893612613439</v>
+        <v>13.0656212552722</v>
       </c>
     </row>
     <row r="426">
@@ -11796,7 +11796,7 @@
         <v>10</v>
       </c>
       <c r="G426" t="n">
-        <v>9.73102915443878</v>
+        <v>8.37946533193485</v>
       </c>
     </row>
     <row r="427">
@@ -11819,7 +11819,7 @@
         <v>6</v>
       </c>
       <c r="G427" t="n">
-        <v>6.04941218318344</v>
+        <v>7.83972485520094</v>
       </c>
     </row>
     <row r="428">
@@ -11842,7 +11842,7 @@
         <v>20</v>
       </c>
       <c r="G428" t="n">
-        <v>9.14704709739769</v>
+        <v>10.0317893200294</v>
       </c>
     </row>
     <row r="429">
@@ -11865,7 +11865,7 @@
         <v>7</v>
       </c>
       <c r="G429" t="n">
-        <v>11.4268360714855</v>
+        <v>12.8884570967438</v>
       </c>
     </row>
     <row r="430">
@@ -11888,7 +11888,7 @@
         <v>6</v>
       </c>
       <c r="G430" t="n">
-        <v>10.7756422753444</v>
+        <v>10.2448546839916</v>
       </c>
     </row>
     <row r="431">
@@ -11911,7 +11911,7 @@
         <v>16</v>
       </c>
       <c r="G431" t="n">
-        <v>5.24263373413182</v>
+        <v>6.44664718440363</v>
       </c>
     </row>
     <row r="432">
@@ -11934,7 +11934,7 @@
         <v>1</v>
       </c>
       <c r="G432" t="n">
-        <v>9.84871424997593</v>
+        <v>9.18755448042987</v>
       </c>
     </row>
     <row r="433">
@@ -11957,7 +11957,7 @@
         <v>15</v>
       </c>
       <c r="G433" t="n">
-        <v>4.01412736008013</v>
+        <v>4.00467920101112</v>
       </c>
     </row>
     <row r="434">
@@ -11980,7 +11980,7 @@
         <v>1</v>
       </c>
       <c r="G434" t="n">
-        <v>7.62617228848447</v>
+        <v>6.31309094782425</v>
       </c>
     </row>
     <row r="435">
@@ -12003,7 +12003,7 @@
         <v>9.43</v>
       </c>
       <c r="G435" t="n">
-        <v>9.24583425324547</v>
+        <v>9.53770492550213</v>
       </c>
     </row>
     <row r="436">
@@ -12026,7 +12026,7 @@
         <v>20.73</v>
       </c>
       <c r="G436" t="n">
-        <v>4.20714847426577</v>
+        <v>5.11984176155535</v>
       </c>
     </row>
     <row r="437">
@@ -12049,7 +12049,7 @@
         <v>13.69</v>
       </c>
       <c r="G437" t="n">
-        <v>2.14135947829077</v>
+        <v>1.76683557075299</v>
       </c>
     </row>
     <row r="438">
@@ -12072,7 +12072,7 @@
         <v>10.45</v>
       </c>
       <c r="G438" t="n">
-        <v>3.72247679685167</v>
+        <v>4.19831994914264</v>
       </c>
     </row>
     <row r="439">
@@ -12095,7 +12095,7 @@
         <v>14.93</v>
       </c>
       <c r="G439" t="n">
-        <v>38.0836717603226</v>
+        <v>32.7726204613057</v>
       </c>
     </row>
     <row r="440">
@@ -12118,7 +12118,7 @@
         <v>13.79</v>
       </c>
       <c r="G440" t="n">
-        <v>1.42421417436487</v>
+        <v>0.72678309572093</v>
       </c>
     </row>
     <row r="441">
@@ -12141,7 +12141,7 @@
         <v>8.06</v>
       </c>
       <c r="G441" t="n">
-        <v>-0.0853736431769638</v>
+        <v>-0.701129062892486</v>
       </c>
     </row>
     <row r="442">
@@ -12164,7 +12164,7 @@
         <v>0.79</v>
       </c>
       <c r="G442" t="n">
-        <v>4.69243787143588</v>
+        <v>4.85450288022813</v>
       </c>
     </row>
     <row r="443">
@@ -12187,7 +12187,7 @@
         <v>0.85</v>
       </c>
       <c r="G443" t="n">
-        <v>1.92280249820427</v>
+        <v>0.88402845078117</v>
       </c>
     </row>
     <row r="444">
@@ -12210,7 +12210,7 @@
         <v>-4.09</v>
       </c>
       <c r="G444" t="n">
-        <v>5.36929548380605</v>
+        <v>4.0685324122299</v>
       </c>
     </row>
     <row r="445">
@@ -12233,7 +12233,7 @@
         <v>-0.74</v>
       </c>
       <c r="G445" t="n">
-        <v>2.56727206550877</v>
+        <v>3.11034645133161</v>
       </c>
     </row>
     <row r="446">
@@ -12256,7 +12256,7 @@
         <v>-1.86</v>
       </c>
       <c r="G446" t="n">
-        <v>4.25779117093147</v>
+        <v>5.884248414691</v>
       </c>
     </row>
     <row r="447">
@@ -12279,7 +12279,7 @@
         <v>-6.6</v>
       </c>
       <c r="G447" t="n">
-        <v>2.67168389416865</v>
+        <v>1.95955459965201</v>
       </c>
     </row>
     <row r="448">
@@ -12302,7 +12302,7 @@
         <v>-5.99</v>
       </c>
       <c r="G448" t="n">
-        <v>4.23214461011769</v>
+        <v>3.12826009578956</v>
       </c>
     </row>
     <row r="449">
@@ -12325,7 +12325,7 @@
         <v>-0.48</v>
       </c>
       <c r="G449" t="n">
-        <v>3.71640028319951</v>
+        <v>5.86721353337999</v>
       </c>
     </row>
     <row r="450">
@@ -12348,7 +12348,7 @@
         <v>874.31</v>
       </c>
       <c r="G450" t="n">
-        <v>269.412213011778</v>
+        <v>239.600896279394</v>
       </c>
     </row>
     <row r="451">
@@ -12371,7 +12371,7 @@
         <v>1757.71</v>
       </c>
       <c r="G451" t="n">
-        <v>-110.249218376157</v>
+        <v>-173.395156101371</v>
       </c>
     </row>
     <row r="452">
@@ -12394,7 +12394,7 @@
         <v>1924.77</v>
       </c>
       <c r="G452" t="n">
-        <v>-729.89767712527</v>
+        <v>-720.664803475432</v>
       </c>
     </row>
     <row r="453">
@@ -12417,7 +12417,7 @@
         <v>274.62</v>
       </c>
       <c r="G453" t="n">
-        <v>-394.471159553067</v>
+        <v>-306.391341088172</v>
       </c>
     </row>
     <row r="454">
@@ -12440,7 +12440,7 @@
         <v>545.54</v>
       </c>
       <c r="G454" t="n">
-        <v>4129.95559574297</v>
+        <v>3081.13925962637</v>
       </c>
     </row>
     <row r="455">
@@ -12463,7 +12463,7 @@
         <v>1276.8</v>
       </c>
       <c r="G455" t="n">
-        <v>-719.105752142025</v>
+        <v>-912.281114435474</v>
       </c>
     </row>
     <row r="456">
@@ -12486,7 +12486,7 @@
         <v>-73.1099999999997</v>
       </c>
       <c r="G456" t="n">
-        <v>-1073.44434234694</v>
+        <v>-1235.44596030541</v>
       </c>
     </row>
     <row r="457">
@@ -12509,7 +12509,7 @@
         <v>171.549999999999</v>
       </c>
       <c r="G457" t="n">
-        <v>-136.684189488658</v>
+        <v>-171.418223255169</v>
       </c>
     </row>
     <row r="458">
@@ -12532,7 +12532,7 @@
         <v>621.64</v>
       </c>
       <c r="G458" t="n">
-        <v>-641.945571030583</v>
+        <v>-756.479668148681</v>
       </c>
     </row>
     <row r="459">
@@ -12555,7 +12555,7 @@
         <v>-1588.06</v>
       </c>
       <c r="G459" t="n">
-        <v>10.7341369804115</v>
+        <v>-183.854911303964</v>
       </c>
     </row>
     <row r="460">
@@ -12578,7 +12578,7 @@
         <v>-845.39</v>
       </c>
       <c r="G460" t="n">
-        <v>-576.522325649745</v>
+        <v>-346.581576080496</v>
       </c>
     </row>
     <row r="461">
@@ -12601,7 +12601,7 @@
         <v>-2646.36</v>
       </c>
       <c r="G461" t="n">
-        <v>78.5321271072972</v>
+        <v>218.83986560574</v>
       </c>
     </row>
     <row r="462">
@@ -12624,7 +12624,7 @@
         <v>-1385.12</v>
       </c>
       <c r="G462" t="n">
-        <v>-100.395292615407</v>
+        <v>-362.833366468705</v>
       </c>
     </row>
     <row r="463">
@@ -12647,7 +12647,7 @@
         <v>-2594.04</v>
       </c>
       <c r="G463" t="n">
-        <v>-87.8004778862409</v>
+        <v>-131.663677540024</v>
       </c>
     </row>
     <row r="464">
@@ -12670,7 +12670,7 @@
         <v>-1268.92</v>
       </c>
       <c r="G464" t="n">
-        <v>-149.152140200605</v>
+        <v>355.071452501061</v>
       </c>
     </row>
     <row r="465">
@@ -12693,7 +12693,7 @@
         <v>517.34</v>
       </c>
       <c r="G465" t="n">
-        <v>636.300754813887</v>
+        <v>570.131759214959</v>
       </c>
     </row>
     <row r="466">
@@ -12716,7 +12716,7 @@
         <v>1517.85</v>
       </c>
       <c r="G466" t="n">
-        <v>242.866821413198</v>
+        <v>182.737570802673</v>
       </c>
     </row>
     <row r="467">
@@ -12739,7 +12739,7 @@
         <v>2790.83</v>
       </c>
       <c r="G467" t="n">
-        <v>-508.343605726035</v>
+        <v>-498.248672888647</v>
       </c>
     </row>
     <row r="468">
@@ -12762,7 +12762,7 @@
         <v>739.459999999999</v>
       </c>
       <c r="G468" t="n">
-        <v>-199.090781077524</v>
+        <v>-136.358577439813</v>
       </c>
     </row>
     <row r="469">
@@ -12785,7 +12785,7 @@
         <v>1179</v>
       </c>
       <c r="G469" t="n">
-        <v>3236.32063209372</v>
+        <v>2433.74469228561</v>
       </c>
     </row>
     <row r="470">
@@ -12808,7 +12808,7 @@
         <v>682.55</v>
       </c>
       <c r="G470" t="n">
-        <v>-339.387340393007</v>
+        <v>-533.11840041531</v>
       </c>
     </row>
     <row r="471">
@@ -12831,7 +12831,7 @@
         <v>35.9499999999998</v>
       </c>
       <c r="G471" t="n">
-        <v>-542.286760950305</v>
+        <v>-764.590410309455</v>
       </c>
     </row>
     <row r="472">
@@ -12854,7 +12854,7 @@
         <v>-171.76</v>
       </c>
       <c r="G472" t="n">
-        <v>100.107487312399</v>
+        <v>359.491581435048</v>
       </c>
     </row>
     <row r="473">
@@ -12877,7 +12877,7 @@
         <v>854.04</v>
       </c>
       <c r="G473" t="n">
-        <v>-389.342632451836</v>
+        <v>-435.663969153908</v>
       </c>
     </row>
     <row r="474">
@@ -12900,7 +12900,7 @@
         <v>-1503.6</v>
       </c>
       <c r="G474" t="n">
-        <v>180.500438421364</v>
+        <v>86.0109245380572</v>
       </c>
     </row>
     <row r="475">
@@ -12923,7 +12923,7 @@
         <v>-88.7199999999993</v>
       </c>
       <c r="G475" t="n">
-        <v>-324.032749917785</v>
+        <v>-196.520206061381</v>
       </c>
     </row>
     <row r="476">
@@ -12946,7 +12946,7 @@
         <v>-2305.05</v>
       </c>
       <c r="G476" t="n">
-        <v>257.062942147617</v>
+        <v>396.099478295108</v>
       </c>
     </row>
     <row r="477">
@@ -12969,7 +12969,7 @@
         <v>-1179.58</v>
       </c>
       <c r="G477" t="n">
-        <v>-67.0144043880098</v>
+        <v>-177.948332386332</v>
       </c>
     </row>
     <row r="478">
@@ -12992,7 +12992,7 @@
         <v>-1491.94</v>
       </c>
       <c r="G478" t="n">
-        <v>55.5996488971181</v>
+        <v>17.2300793733352</v>
       </c>
     </row>
     <row r="479">
@@ -13015,7 +13015,7 @@
         <v>-1081</v>
       </c>
       <c r="G479" t="n">
-        <v>273.42365431024</v>
+        <v>671.506489992852</v>
       </c>
     </row>
     <row r="480">
@@ -13038,7 +13038,7 @@
         <v>1.706</v>
       </c>
       <c r="G480" t="n">
-        <v>2.53946482316585</v>
+        <v>2.38542749845789</v>
       </c>
     </row>
     <row r="481">
@@ -13061,7 +13061,7 @@
         <v>4.218</v>
       </c>
       <c r="G481" t="n">
-        <v>0.61741725331519</v>
+        <v>0.486254663766097</v>
       </c>
     </row>
     <row r="482">
@@ -13084,7 +13084,7 @@
         <v>1.578</v>
       </c>
       <c r="G482" t="n">
-        <v>2.00980141489134</v>
+        <v>1.82732751347613</v>
       </c>
     </row>
     <row r="483">
@@ -13107,7 +13107,7 @@
         <v>3.683</v>
       </c>
       <c r="G483" t="n">
-        <v>2.00796958093846</v>
+        <v>2.34825476360878</v>
       </c>
     </row>
     <row r="484">
@@ -13130,7 +13130,7 @@
         <v>2.983</v>
       </c>
       <c r="G484" t="n">
-        <v>5.99677715369626</v>
+        <v>6.17346264866746</v>
       </c>
     </row>
     <row r="485">
@@ -13153,7 +13153,7 @@
         <v>2.44</v>
       </c>
       <c r="G485" t="n">
-        <v>1.90656601092762</v>
+        <v>3.06141680602093</v>
       </c>
     </row>
     <row r="486">
@@ -13176,7 +13176,7 @@
         <v>3.879</v>
       </c>
       <c r="G486" t="n">
-        <v>1.09438761001709</v>
+        <v>1.79474279495046</v>
       </c>
     </row>
     <row r="487">
@@ -13199,7 +13199,7 @@
         <v>0.579999999999998</v>
       </c>
       <c r="G487" t="n">
-        <v>2.19065433652858</v>
+        <v>1.79291469043293</v>
       </c>
     </row>
     <row r="488">
@@ -13222,7 +13222,7 @@
         <v>-1.918</v>
       </c>
       <c r="G488" t="n">
-        <v>1.48256192844192</v>
+        <v>0.871310053827414</v>
       </c>
     </row>
     <row r="489">
@@ -13245,7 +13245,7 @@
         <v>0.672000000000001</v>
       </c>
       <c r="G489" t="n">
-        <v>2.19214635904057</v>
+        <v>1.94775120593257</v>
       </c>
     </row>
     <row r="490">
@@ -13268,7 +13268,7 @@
         <v>0.352999999999998</v>
       </c>
       <c r="G490" t="n">
-        <v>1.76975123568581</v>
+        <v>1.15163072576018</v>
       </c>
     </row>
     <row r="491">
@@ -13291,7 +13291,7 @@
         <v>5.08900000000001</v>
       </c>
       <c r="G491" t="n">
-        <v>1.0350265864855</v>
+        <v>1.42907888681244</v>
       </c>
     </row>
     <row r="492">
@@ -13314,7 +13314,7 @@
         <v>0.181000000000001</v>
       </c>
       <c r="G492" t="n">
-        <v>0.00687637992375301</v>
+        <v>0.683110028190133</v>
       </c>
     </row>
     <row r="493">
@@ -13337,7 +13337,7 @@
         <v>1.311</v>
       </c>
       <c r="G493" t="n">
-        <v>1.70168232260179</v>
+        <v>1.24430853066286</v>
       </c>
     </row>
     <row r="494">
@@ -13360,7 +13360,7 @@
         <v>2.862</v>
       </c>
       <c r="G494" t="n">
-        <v>1.37922429621286</v>
+        <v>0.658302563907224</v>
       </c>
     </row>
     <row r="495">
@@ -13383,7 +13383,7 @@
         <v>54</v>
       </c>
       <c r="G495" t="n">
-        <v>37.1929354646476</v>
+        <v>45.4988684865343</v>
       </c>
     </row>
     <row r="496">
@@ -13406,7 +13406,7 @@
         <v>83</v>
       </c>
       <c r="G496" t="n">
-        <v>29.1767795891612</v>
+        <v>25.1600100448196</v>
       </c>
     </row>
     <row r="497">
@@ -13429,7 +13429,7 @@
         <v>90</v>
       </c>
       <c r="G497" t="n">
-        <v>24.1906170424567</v>
+        <v>27.5349055283822</v>
       </c>
     </row>
     <row r="498">
@@ -13452,7 +13452,7 @@
         <v>35</v>
       </c>
       <c r="G498" t="n">
-        <v>53.7822533955129</v>
+        <v>52.3750288814785</v>
       </c>
     </row>
     <row r="499">
@@ -13475,7 +13475,7 @@
         <v>5</v>
       </c>
       <c r="G499" t="n">
-        <v>93.3395224579783</v>
+        <v>93.4776028938982</v>
       </c>
     </row>
     <row r="500">
@@ -13498,7 +13498,7 @@
         <v>3</v>
       </c>
       <c r="G500" t="n">
-        <v>24.7290857336161</v>
+        <v>28.0880417699167</v>
       </c>
     </row>
     <row r="501">
@@ -13521,7 +13521,7 @@
         <v>25</v>
       </c>
       <c r="G501" t="n">
-        <v>18.6641733601131</v>
+        <v>24.1229300812773</v>
       </c>
     </row>
     <row r="502">
@@ -13544,7 +13544,7 @@
         <v>72</v>
       </c>
       <c r="G502" t="n">
-        <v>50.3375197373489</v>
+        <v>47.7128203768275</v>
       </c>
     </row>
     <row r="503">
@@ -13567,7 +13567,7 @@
         <v>49</v>
       </c>
       <c r="G503" t="n">
-        <v>35.5101973651342</v>
+        <v>41.0388572469158</v>
       </c>
     </row>
     <row r="504">
@@ -13590,7 +13590,7 @@
         <v>5</v>
       </c>
       <c r="G504" t="n">
-        <v>34.9766210329009</v>
+        <v>41.7633329633098</v>
       </c>
     </row>
     <row r="505">
@@ -13613,7 +13613,7 @@
         <v>62</v>
       </c>
       <c r="G505" t="n">
-        <v>35.1284187523602</v>
+        <v>33.79957215489</v>
       </c>
     </row>
     <row r="506">
@@ -13636,7 +13636,7 @@
         <v>25</v>
       </c>
       <c r="G506" t="n">
-        <v>31.7285587520816</v>
+        <v>2.08909266556991</v>
       </c>
     </row>
     <row r="507">
@@ -13659,7 +13659,7 @@
         <v>18</v>
       </c>
       <c r="G507" t="n">
-        <v>97.5410717889249</v>
+        <v>69.8514757317078</v>
       </c>
     </row>
     <row r="508">
@@ -13682,7 +13682,7 @@
         <v>5</v>
       </c>
       <c r="G508" t="n">
-        <v>54.7042082415315</v>
+        <v>53.3875544762084</v>
       </c>
     </row>
     <row r="509">
@@ -13705,7 +13705,7 @@
         <v>89</v>
       </c>
       <c r="G509" t="n">
-        <v>58.6168554827609</v>
+        <v>45.8556814398153</v>
       </c>
     </row>
     <row r="510">
@@ -13728,7 +13728,7 @@
         <v>5</v>
       </c>
       <c r="G510" t="n">
-        <v>10.3147660796419</v>
+        <v>9.4454609453944</v>
       </c>
     </row>
     <row r="511">
@@ -13751,7 +13751,7 @@
         <v>14</v>
       </c>
       <c r="G511" t="n">
-        <v>0.973126894078598</v>
+        <v>2.56322768435671</v>
       </c>
     </row>
     <row r="512">
@@ -13774,7 +13774,7 @@
         <v>4</v>
       </c>
       <c r="G512" t="n">
-        <v>13.4349103864416</v>
+        <v>12.8858302880222</v>
       </c>
     </row>
     <row r="513">
@@ -13797,7 +13797,7 @@
         <v>11</v>
       </c>
       <c r="G513" t="n">
-        <v>8.82851310547368</v>
+        <v>7.9581091537959</v>
       </c>
     </row>
     <row r="514">
@@ -13820,7 +13820,7 @@
         <v>10</v>
       </c>
       <c r="G514" t="n">
-        <v>15.613112971705</v>
+        <v>15.7854766758341</v>
       </c>
     </row>
     <row r="515">
@@ -13843,7 +13843,7 @@
         <v>23</v>
       </c>
       <c r="G515" t="n">
-        <v>9.41473221283654</v>
+        <v>7.91457773949258</v>
       </c>
     </row>
     <row r="516">
@@ -13866,7 +13866,7 @@
         <v>6</v>
       </c>
       <c r="G516" t="n">
-        <v>8.33042722454857</v>
+        <v>6.75430278847231</v>
       </c>
     </row>
     <row r="517">
@@ -13889,7 +13889,7 @@
         <v>20</v>
       </c>
       <c r="G517" t="n">
-        <v>8.08097966063268</v>
+        <v>6.88334584607214</v>
       </c>
     </row>
     <row r="518">
@@ -13912,7 +13912,7 @@
         <v>7</v>
       </c>
       <c r="G518" t="n">
-        <v>13.7754182774119</v>
+        <v>12.6423037905917</v>
       </c>
     </row>
     <row r="519">
@@ -13935,7 +13935,7 @@
         <v>6</v>
       </c>
       <c r="G519" t="n">
-        <v>10.3882054067286</v>
+        <v>11.2408193348312</v>
       </c>
     </row>
     <row r="520">
@@ -13958,7 +13958,7 @@
         <v>16</v>
       </c>
       <c r="G520" t="n">
-        <v>12.4136749930243</v>
+        <v>16.1628089154329</v>
       </c>
     </row>
     <row r="521">
@@ -13981,7 +13981,7 @@
         <v>1</v>
       </c>
       <c r="G521" t="n">
-        <v>11.3766042930283</v>
+        <v>11.9114240602969</v>
       </c>
     </row>
     <row r="522">
@@ -14004,7 +14004,7 @@
         <v>15</v>
       </c>
       <c r="G522" t="n">
-        <v>8.84046197278529</v>
+        <v>8.26434839202819</v>
       </c>
     </row>
     <row r="523">
@@ -14027,7 +14027,7 @@
         <v>1</v>
       </c>
       <c r="G523" t="n">
-        <v>9.06447024473779</v>
+        <v>8.91103617408106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>